<commit_message>
vault backup: 2026-10-09 10:40:18
</commit_message>
<xml_diff>
--- a/WLS-VN-live.xlsx
+++ b/WLS-VN-live.xlsx
@@ -624,7 +624,7 @@
       <c r="D5" s="3" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -696,7 +696,7 @@
       <c r="D8" s="3" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -720,7 +720,7 @@
       <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -944,7 +944,7 @@
       <c r="D18" s="3" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -992,7 +992,7 @@
       <c r="D20" s="3" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1132,7 +1132,7 @@
       <c r="D25" s="3" t="inlineStr"/>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -1252,7 +1252,7 @@
       <c r="D30" s="3" t="inlineStr"/>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -1276,7 +1276,7 @@
       <c r="D31" s="3" t="inlineStr"/>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -1732,7 +1732,7 @@
       <c r="D50" s="3" t="inlineStr"/>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
@@ -1776,16 +1776,8 @@
           <t>103.82.194.3:443</t>
         </is>
       </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
+      <c r="C52" s="3" t="inlineStr"/>
+      <c r="D52" s="3" t="inlineStr"/>
       <c r="E52" s="3" t="inlineStr">
         <is>
           <t>Da Nang</t>
@@ -2025,7 +2017,7 @@
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>越南邮政电信集团</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
@@ -2293,7 +2285,7 @@
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>越南邮政电信集团</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
@@ -2403,7 +2395,7 @@
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>console-open;T3-open</t>
+          <t>console-open</t>
         </is>
       </c>
       <c r="E74" s="6" t="inlineStr">
@@ -2753,7 +2745,7 @@
       </c>
       <c r="F86" s="6" t="inlineStr">
         <is>
-          <t>越南电信</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2769,7 @@
       </c>
       <c r="F87" s="6" t="inlineStr">
         <is>
-          <t>越南电信</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
@@ -3069,7 +3061,7 @@
       </c>
       <c r="F98" s="6" t="inlineStr">
         <is>
-          <t>越南邮政电信集团</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
@@ -3165,7 +3157,7 @@
       </c>
       <c r="F102" s="6" t="inlineStr">
         <is>
-          <t>越南邮政电信集团</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
@@ -3340,7 +3332,7 @@
       <c r="D109" s="6" t="inlineStr"/>
       <c r="E109" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F109" s="6" t="inlineStr">

</xml_diff>

<commit_message>
vault backup: 2026-10-09 10:55:26
</commit_message>
<xml_diff>
--- a/WLS-VN-live.xlsx
+++ b/WLS-VN-live.xlsx
@@ -1012,7 +1012,11 @@
           <t>113.161.81.238:8081</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
           <t>T3-open</t>

</xml_diff>

<commit_message>
vault backup: 2026-10-09 11:10:36
</commit_message>
<xml_diff>
--- a/WLS-VN-live.xlsx
+++ b/WLS-VN-live.xlsx
@@ -529,9 +529,9 @@
           <t>10.3.6.0</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>T3-open</t>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -556,11 +556,7 @@
           <t>113.160.129.228:9001</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
+      <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr">
         <is>
           <t>T3-open</t>
@@ -1540,8 +1536,16 @@
           <t>42.115.41.28:443</t>
         </is>
       </c>
-      <c r="C42" s="3" t="inlineStr"/>
-      <c r="D42" s="3" t="inlineStr"/>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>12.2.1.3.0</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -1780,8 +1784,16 @@
           <t>103.82.194.3:443</t>
         </is>
       </c>
-      <c r="C52" s="3" t="inlineStr"/>
-      <c r="D52" s="3" t="inlineStr"/>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
           <t>Da Nang</t>

</xml_diff>

<commit_message>
vault backup: 2026-10-09 11:56:03
</commit_message>
<xml_diff>
--- a/WLS-VN-live.xlsx
+++ b/WLS-VN-live.xlsx
@@ -10,7 +10,7 @@
     <sheet name="WLS VN (live)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WLS VN (live)'!$A$1:$F$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WLS VN (live)'!$A$1:$F$137</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F109"/>
+  <dimension ref="A1:F137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -636,12 +636,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>https://rsaweb.mps.gov.vn</t>
+          <t>http://xbi.xteco.org</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>42.1.75.65:443</t>
+          <t>27.71.231.120:80</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
@@ -653,19 +653,19 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>MOBIFONE Corporation</t>
+          <t>CHT Compamy Ltd</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>https://hochieu.xuatnhapcanh.gov.vn</t>
+          <t>https://xbi.xteco.org</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>42.112.168.100:443</t>
+          <t>27.71.231.120:443</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr"/>
@@ -677,19 +677,19 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>CHT Compamy Ltd</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>https://quanlyluutru.xuatnhapcanh.gov.vn</t>
+          <t>https://rsaweb.mps.gov.vn</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>42.112.168.116:443</t>
+          <t>42.1.75.65:443</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
@@ -701,31 +701,23 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>MOBIFONE Corporation</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>https://orabi.kimdental.vn</t>
+          <t>https://hochieu.xuatnhapcanh.gov.vn</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>42.115.41.28:443</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>12.2.1.3.0</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
+          <t>42.112.168.100:443</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -740,12 +732,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>http://dvc.vst.mof.gov.vn</t>
+          <t>https://quanlyluutru.xuatnhapcanh.gov.vn</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.40:80</t>
+          <t>42.112.168.116:443</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
@@ -757,23 +749,31 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>https://dvc.vst.mof.gov.vn</t>
+          <t>https://orabi.kimdental.vn</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.40:443</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr"/>
-      <c r="D12" s="3" t="inlineStr"/>
+          <t>42.115.41.28:443</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>12.2.1.3.0</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -781,19 +781,19 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>http://dvctn.vst.mof.gov.vn</t>
+          <t>http://dvc.vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.41:80</t>
+          <t>45.120.230.40:80</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
@@ -812,12 +812,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>https://dvctn.vst.mof.gov.vn</t>
+          <t>https://dvc.vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.41:443</t>
+          <t>45.120.230.40:443</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr"/>
@@ -836,12 +836,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>http://vst.mof.gov.vn</t>
+          <t>http://dvctn.vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.45:80</t>
+          <t>45.120.230.41:80</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
@@ -860,12 +860,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>http://bctcnn.vst.mof.gov.vn</t>
+          <t>https://dvctn.vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.50:80</t>
+          <t>45.120.230.41:443</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr"/>
@@ -884,12 +884,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>https://bctcnn.vst.mof.gov.vn</t>
+          <t>http://vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.50:443</t>
+          <t>45.120.230.45:80</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
@@ -908,12 +908,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>http://tracuudvc.vst.mof.gov.vn</t>
+          <t>http://bctcnn.vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.51:80</t>
+          <t>45.120.230.50:80</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr"/>
@@ -932,12 +932,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>https://tracuudvc.vst.mof.gov.vn</t>
+          <t>https://bctcnn.vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.51:443</t>
+          <t>45.120.230.50:443</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr"/>
@@ -956,12 +956,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>http://pus.customs.gov.vn</t>
+          <t>http://tracuudvc.vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>58.186.80.48:80</t>
+          <t>45.120.230.51:80</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr"/>
@@ -973,19 +973,19 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>Creative Communication Vietnam Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>https://pus.customs.gov.vn</t>
+          <t>https://tracuudvc.vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>58.186.80.48:443</t>
+          <t>45.120.230.51:443</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr"/>
@@ -997,19 +997,19 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>Creative Communication Vietnam Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>http://ids.ssc.gov.vn</t>
+          <t>http://tongcuc.hotrokythuat.asia:8080</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>103.3.252.106:80</t>
+          <t>45.122.253.178:8080</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr"/>
@@ -1021,43 +1021,39 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>https://ids.ssc.gov.vn</t>
+          <t>http://dichvucong.danang.vn</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>103.3.252.106:443</t>
+          <t>49.156.52.22:80</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr"/>
       <c r="D23" s="3" t="inlineStr"/>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
-        </is>
-      </c>
+          <t>Da Nang</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>https://congbothongtin.ssc.gov.vn</t>
+          <t>http://pus.customs.gov.vn</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>103.3.252.107:443</t>
+          <t>58.186.80.48:80</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr"/>
@@ -1069,19 +1065,19 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>https://ssc.gov.vn</t>
+          <t>https://pus.customs.gov.vn</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>103.3.252.109:443</t>
+          <t>58.186.80.48:443</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr"/>
@@ -1093,19 +1089,19 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>https://cims.hnx.vn</t>
+          <t>http://ids.ssc.gov.vn</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>103.9.212.43:443</t>
+          <t>103.3.252.106:80</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr"/>
@@ -1117,99 +1113,91 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>HaNoi Stock Exchange</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>https://www.xsmb360.com</t>
+          <t>https://ids.ssc.gov.vn</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>103.82.194.3:443</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
+          <t>103.3.252.106:443</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Da Nang</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>http://idm.homecredit.vn</t>
+          <t>http://congbothongtin.ssc.gov.vn</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>103.111.244.73:80</t>
+          <t>103.3.252.107:80</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr"/>
       <c r="D28" s="3" t="inlineStr"/>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Home Credit Viet nam Finance Company Limited</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>https://idm.homecredit.vn</t>
+          <t>https://congbothongtin.ssc.gov.vn</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>103.111.244.73:443</t>
+          <t>103.3.252.107:443</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr"/>
       <c r="D29" s="3" t="inlineStr"/>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Home Credit Viet nam Finance Company Limited</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>https://www.vinpro.net</t>
+          <t>https://ssc.gov.vn</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>103.238.209.204:443</t>
+          <t>103.3.252.109:443</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr"/>
@@ -1221,155 +1209,123 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>VINGROUP JOINT STOCK COMPANY</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>http://apvs1.dlp.com.tw:7001</t>
+          <t>http://cims.hnx.vn</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>113.160.129.228:7001</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>103.9.212.43:80</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Hai Duong</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>HaNoi Stock Exchange</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>http://apvs1.dlp.com.tw:9001</t>
+          <t>https://cims.hnx.vn</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>113.160.129.228:9001</t>
+          <t>103.9.212.43:443</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr"/>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+      <c r="D32" s="3" t="inlineStr"/>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Hai Duong</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>HaNoi Stock Exchange</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>http://apvs1.dlp.com.tw:9002</t>
+          <t>http://hse.vn</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>113.160.129.228:9002</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>103.9.212.46:80</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Hai Duong</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>VNPT Corp</t>
-        </is>
-      </c>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>http://www.dtsweb.tech:8081</t>
+          <t>https://www.xsmb360.com</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>113.161.81.238:8081</t>
+          <t>103.82.194.3:443</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>T3-open</t>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Da Nang</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>http://www.dtsweb.tech:9001</t>
+          <t>http://idm.homecredit.vn</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>113.161.81.238:9001</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>103.111.244.73:80</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
       <c r="E35" s="3" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
@@ -1377,75 +1333,67 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Home Credit Viet nam Finance Company Limited</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>http://www.hddt.agimexpharm.com:8082</t>
+          <t>https://idm.homecredit.vn</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>113.161.212.113:8082</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>103.111.244.73:443</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr"/>
+      <c r="D36" s="3" t="inlineStr"/>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Long Xuyen</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Home Credit Viet nam Finance Company Limited</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>https://pritos.cloud:3068</t>
+          <t>https://www.vinpro.net</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>115.75.20.142:3068</t>
+          <t>103.238.209.204:443</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr"/>
       <c r="D37" s="3" t="inlineStr"/>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Thi Tran Long Dien</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>VINGROUP JOINT STOCK COMPANY</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>http://trienlamso.ictquangtri.vn</t>
+          <t>https://eoffice.myvnc.com</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>117.122.125.107:80</t>
+          <t>113.160.48.99:443</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr"/>
@@ -1457,50 +1405,66 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Internet Network Information Center</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>https://euroeximbank.com.vn</t>
+          <t>http://apvs1.dlp.com.tw:7001</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>117.122.125.107:443</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr"/>
+          <t>113.160.129.228:7001</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Hai Duong</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Internet Network Information Center</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>http://capcaohcm.toaan.gov.vn</t>
+          <t>http://apvs1.dlp.com.tw:9001</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>123.30.24.180:80</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr"/>
-      <c r="D40" s="3" t="inlineStr"/>
+          <t>113.160.129.228:9001</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>T3-open</t>
+        </is>
+      </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Hai Duong</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -1512,19 +1476,27 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>https://mla.toaan.gov.vn</t>
+          <t>http://apvs1.dlp.com.tw:9002</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>123.30.24.180:443</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr"/>
+          <t>113.160.129.228:9002</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>T3-open</t>
+        </is>
+      </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Hai Duong</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -1536,19 +1508,27 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>https://cskh.temxacthuc.vn:8081</t>
+          <t>http://www.dtsweb.tech:8081</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>123.30.208.19:8081</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr"/>
-      <c r="D42" s="3" t="inlineStr"/>
+          <t>113.161.81.238:8081</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>T3-open</t>
+        </is>
+      </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
@@ -1560,60 +1540,76 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>http://gmobi.vn</t>
+          <t>http://www.dtsweb.tech:9001</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>123.31.31.126:80</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr"/>
+          <t>113.161.81.238:9001</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>T3-open</t>
+        </is>
+      </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>http://csdlgiaquocgia.mof.gov.vn</t>
+          <t>http://www.hddt.agimexpharm.com:8082</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>182.236.113.46:80</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr"/>
-      <c r="D44" s="3" t="inlineStr"/>
+          <t>113.161.212.113:8082</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>T3-open</t>
+        </is>
+      </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Long Xuyen</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Department of Information Technology and Digital Transformation - Ministry of Finance</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>https://csdlgiaquocgia.mof.gov.vn</t>
+          <t>http://webdisk.sophattai.com:8080</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>182.236.113.46:443</t>
+          <t>113.185.19.167:8080</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr"/>
@@ -1625,67 +1621,63 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Department of Information Technology and Digital Transformation - Ministry of Finance</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>http://thongbaotenmien.vn</t>
+          <t>https://pritos.cloud:3068</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>203.119.73.12:80</t>
+          <t>115.75.20.142:3068</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr"/>
       <c r="D46" s="3" t="inlineStr"/>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Thi Tran Long Dien</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Internet network information center (VNNIC)</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>https://thongbaotenmien.vn</t>
+          <t>http://thi.moet.gov.vn</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>203.119.73.12:443</t>
+          <t>115.146.127.162:80</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr"/>
       <c r="D47" s="3" t="inlineStr"/>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="inlineStr">
-        <is>
-          <t>Vietnam Internet network information center (VNNIC)</t>
-        </is>
-      </c>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>http://sso.vietinbank.vn</t>
+          <t>https://thi.moet.gov.vn</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>203.189.29.33:80</t>
+          <t>115.146.127.162:443</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr"/>
@@ -1695,21 +1687,17 @@
           <t>Hanoi</t>
         </is>
       </c>
-      <c r="F48" s="3" t="inlineStr">
-        <is>
-          <t>VIETINBANK-VN</t>
-        </is>
-      </c>
+      <c r="F48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>https://sso.vietinbank.vn</t>
+          <t>http://trienlamso.ictquangtri.vn</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>203.189.29.33:443</t>
+          <t>117.122.125.107:80</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr"/>
@@ -1721,658 +1709,610 @@
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>VIETINBANK-VN</t>
+          <t>Vietnam Internet Network Information Center</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>http://htttsv.hoasen.edu.vn</t>
+          <t>https://euroeximbank.com.vn</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>203.205.57.225:80</t>
+          <t>117.122.125.107:443</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr"/>
       <c r="D50" s="3" t="inlineStr"/>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>CMC Telecom Infrastructure Company</t>
+          <t>Vietnam Internet Network Information Center</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>https://htttsv.hoasen.edu.vn</t>
+          <t>http://capcaohcm.toaan.gov.vn</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>203.205.57.225:443</t>
+          <t>123.30.24.180:80</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr"/>
       <c r="D51" s="3" t="inlineStr"/>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>CMC Telecom Infrastructure Company</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>http://erptest.hoasen.edu.vn:80</t>
+          <t>https://mla.toaan.gov.vn</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
+          <t>123.30.24.180:443</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr"/>
+      <c r="D52" s="3" t="inlineStr"/>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>https://cskh.temxacthuc.vn:8081</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>123.30.208.19:8081</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr"/>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>http://www.topteen.vn</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>123.30.208.25:80</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr"/>
+      <c r="D54" s="3" t="inlineStr"/>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>http://gmobi.vn</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>123.31.31.126:80</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr"/>
+      <c r="D55" s="3" t="inlineStr"/>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>http://cskh.temdientu.vn</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>123.31.41.93:80</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr"/>
+      <c r="D56" s="3" t="inlineStr"/>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>http://csdlgiaquocgia.mof.gov.vn</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>182.236.113.46:80</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr"/>
+      <c r="D57" s="3" t="inlineStr"/>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Department of Information Technology and Digital Transformation - Ministry of Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>https://csdlgiaquocgia.mof.gov.vn</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>182.236.113.46:443</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr"/>
+      <c r="D58" s="3" t="inlineStr"/>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>Department of Information Technology and Digital Transformation - Ministry of Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>http://thongbaotenmien.vn</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>203.119.73.12:80</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr"/>
+      <c r="D59" s="3" t="inlineStr"/>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>Vietnam Internet network information center (VNNIC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>https://thongbaotenmien.vn</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>203.119.73.12:443</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr"/>
+      <c r="D60" s="3" t="inlineStr"/>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>Vietnam Internet network information center (VNNIC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>http://qlahs.vksndtc.gov.vn</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>203.162.255.5:80</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr"/>
+      <c r="D61" s="3" t="inlineStr"/>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>http://chuyentien.vietinbank.vn</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>203.189.28.86:80</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr"/>
+      <c r="D62" s="3" t="inlineStr"/>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>VIETINBANK</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>http://sso.vietinbank.vn</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>203.189.29.33:80</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr"/>
+      <c r="D63" s="3" t="inlineStr"/>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>VIETINBANK-VN</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>https://sso.vietinbank.vn</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>203.189.29.33:443</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr"/>
+      <c r="D64" s="3" t="inlineStr"/>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>VIETINBANK-VN</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>http://htttsv.hoasen.edu.vn</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>203.205.57.225:80</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr"/>
+      <c r="D65" s="3" t="inlineStr"/>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>CMC Telecom Infrastructure Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>https://htttsv.hoasen.edu.vn</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>203.205.57.225:443</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr"/>
+      <c r="D66" s="3" t="inlineStr"/>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>CMC Telecom Infrastructure Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>http://erpbk.hoasen.edu.vn</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
           <t>203.205.57.226:80</t>
         </is>
       </c>
-      <c r="C52" s="3" t="inlineStr">
+      <c r="C67" s="3" t="inlineStr">
         <is>
           <t>10.3.4.0</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
+      <c r="D67" s="4" t="inlineStr">
         <is>
           <t>console-open</t>
         </is>
       </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
         <is>
           <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
-        <is>
-          <t>http://14.225.11.33:9001</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
-        <is>
-          <t>14.225.11.33:9001</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
-      <c r="E53" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
-        <is>
-          <t>http://14.238.41.12:80</t>
-        </is>
-      </c>
-      <c r="B54" s="6" t="inlineStr">
-        <is>
-          <t>14.238.41.12:80</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="inlineStr"/>
-      <c r="D54" s="6" t="inlineStr"/>
-      <c r="E54" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>http://cms.mebongda.net</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>210.211.99.108:80</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr"/>
+      <c r="D68" s="3" t="inlineStr"/>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>CHT Compamy Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>http://static.ketquasieutoc.com:8080</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>210.211.99.108:8080</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr"/>
+      <c r="D69" s="3" t="inlineStr"/>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>CHT Compamy Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>http://mobilaw.vn</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>210.211.99.130:80</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr"/>
+      <c r="D70" s="3" t="inlineStr"/>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>http://m.xosothongminh.vn</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>210.211.99.133:80</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr"/>
+      <c r="D71" s="3" t="inlineStr"/>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>http://rvt.kenhnhac.vn</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>210.211.99.174:80</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr"/>
+      <c r="D72" s="3" t="inlineStr"/>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>CHT Compamy Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>http://dvc-kbnn.fintechviet.vn</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>222.252.98.4:80</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr"/>
+      <c r="D73" s="3" t="inlineStr"/>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>https://14.238.93.114:9184</t>
-        </is>
-      </c>
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>14.238.93.114:9184</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="inlineStr"/>
-      <c r="D55" s="6" t="inlineStr"/>
-      <c r="E55" s="6" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="inlineStr">
-        <is>
-          <t>VNPT Corp</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t>http://14.241.253.96:8081</t>
-        </is>
-      </c>
-      <c r="B56" s="6" t="inlineStr">
-        <is>
-          <t>14.241.253.96:8081</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="inlineStr"/>
-      <c r="D56" s="6" t="inlineStr"/>
-      <c r="E56" s="6" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="inlineStr">
-        <is>
-          <t>VNPT Corp</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
-        <is>
-          <t>http://14.241.253.96:8082</t>
-        </is>
-      </c>
-      <c r="B57" s="6" t="inlineStr">
-        <is>
-          <t>14.241.253.96:8082</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="inlineStr"/>
-      <c r="D57" s="6" t="inlineStr"/>
-      <c r="E57" s="6" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="inlineStr">
-        <is>
-          <t>VNPT Corp</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
-        <is>
-          <t>https://14.248.84.7:443</t>
-        </is>
-      </c>
-      <c r="B58" s="6" t="inlineStr">
-        <is>
-          <t>14.248.84.7:443</t>
-        </is>
-      </c>
-      <c r="C58" s="6" t="inlineStr"/>
-      <c r="D58" s="6" t="inlineStr"/>
-      <c r="E58" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="inlineStr">
-        <is>
-          <t>VNPT Corp</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t>http://27.72.123.124:8001</t>
-        </is>
-      </c>
-      <c r="B59" s="6" t="inlineStr">
-        <is>
-          <t>27.72.123.124:8001</t>
-        </is>
-      </c>
-      <c r="C59" s="6" t="inlineStr"/>
-      <c r="D59" s="6" t="inlineStr"/>
-      <c r="E59" s="6" t="inlineStr">
-        <is>
-          <t>Sa Pa</t>
-        </is>
-      </c>
-      <c r="F59" s="6" t="inlineStr">
-        <is>
-          <t>Viettel Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
-        <is>
-          <t>http://27.72.123.124:8003</t>
-        </is>
-      </c>
-      <c r="B60" s="6" t="inlineStr">
-        <is>
-          <t>27.72.123.124:8003</t>
-        </is>
-      </c>
-      <c r="C60" s="6" t="inlineStr"/>
-      <c r="D60" s="6" t="inlineStr"/>
-      <c r="E60" s="6" t="inlineStr">
-        <is>
-          <t>Ha Long</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="inlineStr">
-        <is>
-          <t>Viettel Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
-        <is>
-          <t>https://42.115.41.27:443</t>
-        </is>
-      </c>
-      <c r="B61" s="6" t="inlineStr">
-        <is>
-          <t>42.115.41.27:443</t>
-        </is>
-      </c>
-      <c r="C61" s="6" t="inlineStr"/>
-      <c r="D61" s="6" t="inlineStr"/>
-      <c r="E61" s="6" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
-      <c r="F61" s="6" t="inlineStr">
-        <is>
-          <t>FPT Telecom Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
-        <is>
-          <t>http://42.118.60.193:7001</t>
-        </is>
-      </c>
-      <c r="B62" s="6" t="inlineStr">
-        <is>
-          <t>42.118.60.193:7001</t>
-        </is>
-      </c>
-      <c r="C62" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D62" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
-      <c r="E62" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="inlineStr">
-        <is>
-          <t>FPT Telecom Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
-        <is>
-          <t>https://45.120.230.45</t>
-        </is>
-      </c>
-      <c r="B63" s="6" t="inlineStr">
-        <is>
-          <t>45.120.230.45:443</t>
-        </is>
-      </c>
-      <c r="C63" s="6" t="inlineStr"/>
-      <c r="D63" s="6" t="inlineStr"/>
-      <c r="E63" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F63" s="6" t="inlineStr">
-        <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
-        <is>
-          <t>http://49.213.88.170:7001</t>
-        </is>
-      </c>
-      <c r="B64" s="6" t="inlineStr">
-        <is>
-          <t>49.213.88.170:7001</t>
-        </is>
-      </c>
-      <c r="C64" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D64" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="inlineStr">
-        <is>
-          <t>VNG Corporation</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="5" t="inlineStr">
-        <is>
-          <t>https://103.3.252.106:7002</t>
-        </is>
-      </c>
-      <c r="B65" s="6" t="inlineStr">
-        <is>
-          <t>103.3.252.106:7002</t>
-        </is>
-      </c>
-      <c r="C65" s="6" t="inlineStr"/>
-      <c r="D65" s="6" t="inlineStr"/>
-      <c r="E65" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="inlineStr">
-        <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
-        <is>
-          <t>http://103.3.252.107:80</t>
-        </is>
-      </c>
-      <c r="B66" s="6" t="inlineStr">
-        <is>
-          <t>103.3.252.107:80</t>
-        </is>
-      </c>
-      <c r="C66" s="6" t="inlineStr"/>
-      <c r="D66" s="6" t="inlineStr"/>
-      <c r="E66" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F66" s="6" t="inlineStr">
-        <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="5" t="inlineStr">
-        <is>
-          <t>https://103.3.252.107:7002</t>
-        </is>
-      </c>
-      <c r="B67" s="6" t="inlineStr">
-        <is>
-          <t>103.3.252.107:7002</t>
-        </is>
-      </c>
-      <c r="C67" s="6" t="inlineStr"/>
-      <c r="D67" s="6" t="inlineStr"/>
-      <c r="E67" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F67" s="6" t="inlineStr">
-        <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="5" t="inlineStr">
-        <is>
-          <t>http://103.3.252.109:80</t>
-        </is>
-      </c>
-      <c r="B68" s="6" t="inlineStr">
-        <is>
-          <t>103.3.252.109:80</t>
-        </is>
-      </c>
-      <c r="C68" s="6" t="inlineStr"/>
-      <c r="D68" s="6" t="inlineStr"/>
-      <c r="E68" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F68" s="6" t="inlineStr">
-        <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="inlineStr">
-        <is>
-          <t>http://103.3.252.133:80</t>
-        </is>
-      </c>
-      <c r="B69" s="6" t="inlineStr">
-        <is>
-          <t>103.3.252.133:80</t>
-        </is>
-      </c>
-      <c r="C69" s="6" t="inlineStr"/>
-      <c r="D69" s="6" t="inlineStr"/>
-      <c r="E69" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F69" s="6" t="inlineStr">
-        <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="5" t="inlineStr">
-        <is>
-          <t>http://103.9.212.43:80</t>
-        </is>
-      </c>
-      <c r="B70" s="6" t="inlineStr">
-        <is>
-          <t>103.9.212.43:80</t>
-        </is>
-      </c>
-      <c r="C70" s="6" t="inlineStr"/>
-      <c r="D70" s="6" t="inlineStr"/>
-      <c r="E70" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F70" s="6" t="inlineStr">
-        <is>
-          <t>HaNoi Stock Exchange</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="5" t="inlineStr">
-        <is>
-          <t>http://103.9.213.43:80</t>
-        </is>
-      </c>
-      <c r="B71" s="6" t="inlineStr">
-        <is>
-          <t>103.9.213.43:80</t>
-        </is>
-      </c>
-      <c r="C71" s="6" t="inlineStr"/>
-      <c r="D71" s="6" t="inlineStr"/>
-      <c r="E71" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F71" s="6" t="inlineStr">
-        <is>
-          <t>HaNoi Stock Exchange</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="5" t="inlineStr">
-        <is>
-          <t>http://103.82.192.168</t>
-        </is>
-      </c>
-      <c r="B72" s="6" t="inlineStr">
-        <is>
-          <t>103.82.192.168:80</t>
-        </is>
-      </c>
-      <c r="C72" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D72" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
-      <c r="E72" s="6" t="inlineStr">
-        <is>
-          <t>Da Nang</t>
-        </is>
-      </c>
-      <c r="F72" s="6" t="inlineStr">
-        <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="5" t="inlineStr">
-        <is>
-          <t>https://103.82.192.168</t>
-        </is>
-      </c>
-      <c r="B73" s="6" t="inlineStr">
-        <is>
-          <t>103.82.192.168:443</t>
-        </is>
-      </c>
-      <c r="C73" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D73" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
-      <c r="E73" s="6" t="inlineStr">
-        <is>
-          <t>Da Nang</t>
-        </is>
-      </c>
-      <c r="F73" s="6" t="inlineStr">
-        <is>
-          <t>CLOUDFLY CORPORATION</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>http://103.82.194.3</t>
+          <t>http://14.225.11.33:9001</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>103.82.194.3:80</t>
+          <t>14.225.11.33:9001</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D74" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>T3-open</t>
         </is>
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
-          <t>Da Nang</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
@@ -2384,20 +2324,16 @@
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>https://103.120.242.145:8081</t>
+          <t>http://14.238.41.12:80</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>103.120.242.145:8081</t>
+          <t>14.238.41.12:80</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr"/>
-      <c r="D75" s="6" t="inlineStr">
-        <is>
-          <t>console-403</t>
-        </is>
-      </c>
+      <c r="D75" s="6" t="inlineStr"/>
       <c r="E75" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -2412,12 +2348,12 @@
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>https://103.150.240.14:443</t>
+          <t>https://14.238.93.114:9184</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>103.150.240.14:443</t>
+          <t>14.238.93.114:9184</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr"/>
@@ -2429,159 +2365,143 @@
       </c>
       <c r="F76" s="6" t="inlineStr">
         <is>
-          <t>INTELLIGENCE INFORMATION SYSTEM CO, LTD</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>http://103.238.209.174</t>
+          <t>http://14.241.253.96:8081</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>103.238.209.174:80</t>
+          <t>14.241.253.96:8081</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr"/>
       <c r="D77" s="6" t="inlineStr"/>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F77" s="6" t="inlineStr">
         <is>
-          <t>VINGROUP JOINT STOCK COMPANY</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>https://103.238.209.174</t>
+          <t>http://14.241.253.96:8082</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>103.238.209.174:443</t>
+          <t>14.241.253.96:8082</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr"/>
       <c r="D78" s="6" t="inlineStr"/>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F78" s="6" t="inlineStr">
         <is>
-          <t>VINGROUP JOINT STOCK COMPANY</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>https://112.109.89.131</t>
+          <t>https://14.248.84.7:443</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>112.109.89.131:443</t>
+          <t>14.248.84.7:443</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr"/>
       <c r="D79" s="6" t="inlineStr"/>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F79" s="6" t="inlineStr">
         <is>
-          <t>Minh Tu Telecom Limited Company</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>http://113.160.181.154:8001</t>
+          <t>http://27.72.123.124:8001</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>113.160.181.154:8001</t>
+          <t>27.72.123.124:8001</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr"/>
       <c r="D80" s="6" t="inlineStr"/>
       <c r="E80" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Sa Pa</t>
         </is>
       </c>
       <c r="F80" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>http://113.160.201.159:7001</t>
+          <t>http://27.72.123.124:8003</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>113.160.201.159:7001</t>
-        </is>
-      </c>
-      <c r="C81" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D81" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>27.72.123.124:8003</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr"/>
+      <c r="D81" s="6" t="inlineStr"/>
       <c r="E81" s="6" t="inlineStr">
         <is>
-          <t>Thai Binh</t>
+          <t>Ha Long</t>
         </is>
       </c>
       <c r="F81" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>http://113.161.43.248:9001</t>
+          <t>https://42.115.41.27:443</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>113.161.43.248:9001</t>
-        </is>
-      </c>
-      <c r="C82" s="6" t="inlineStr">
-        <is>
-          <t>14.1.2.0.0</t>
-        </is>
-      </c>
-      <c r="D82" s="6" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>42.115.41.27:443</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr"/>
+      <c r="D82" s="6" t="inlineStr"/>
       <c r="E82" s="6" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
@@ -2589,19 +2509,19 @@
       </c>
       <c r="F82" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>http://113.163.187.3:27001</t>
+          <t>http://42.118.60.193:7001</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>113.163.187.3:27001</t>
+          <t>42.118.60.193:7001</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
@@ -2616,24 +2536,24 @@
       </c>
       <c r="E83" s="6" t="inlineStr">
         <is>
-          <t>Phan Rang-Thap Cham</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F83" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>http://113.185.0.60:8080</t>
+          <t>https://45.120.230.45</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>113.185.0.60:8080</t>
+          <t>45.120.230.45:443</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr"/>
@@ -2645,59 +2565,55 @@
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Creative Communication Vietnam Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>http://113.185.19.167:8080</t>
+          <t>http://49.213.88.170:7001</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>113.185.19.167:8080</t>
-        </is>
-      </c>
-      <c r="C85" s="6" t="inlineStr"/>
-      <c r="D85" s="6" t="inlineStr">
-        <is>
-          <t>console-403</t>
+          <t>49.213.88.170:7001</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
         </is>
       </c>
       <c r="E85" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F85" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>VNG Corporation</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>http://117.4.32.40:1111</t>
+          <t>https://103.3.252.106:7002</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>117.4.32.40:1111</t>
-        </is>
-      </c>
-      <c r="C86" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D86" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>103.3.252.106:7002</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="inlineStr"/>
+      <c r="D86" s="6" t="inlineStr"/>
       <c r="E86" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -2705,31 +2621,23 @@
       </c>
       <c r="F86" s="6" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>http://117.4.241.247:1112</t>
+          <t>https://103.3.252.107:7002</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>117.4.241.247:1112</t>
-        </is>
-      </c>
-      <c r="C87" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D87" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>103.3.252.107:7002</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr"/>
+      <c r="D87" s="6" t="inlineStr"/>
       <c r="E87" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -2737,75 +2645,67 @@
       </c>
       <c r="F87" s="6" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>https://118.69.32.193:3068</t>
+          <t>http://103.3.252.109:80</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>118.69.32.193:3068</t>
+          <t>103.3.252.109:80</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr"/>
       <c r="D88" s="6" t="inlineStr"/>
       <c r="E88" s="6" t="inlineStr">
         <is>
-          <t>Thu Dau Mot</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F88" s="6" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>http://118.69.182.224:9079</t>
+          <t>http://103.3.252.133</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>118.69.182.224:9079</t>
-        </is>
-      </c>
-      <c r="C89" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D89" s="6" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>103.3.252.133:80</t>
+        </is>
+      </c>
+      <c r="C89" s="6" t="inlineStr"/>
+      <c r="D89" s="6" t="inlineStr"/>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t>Bien Hoa</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F89" s="6" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>http://123.30.208.19:80</t>
+          <t>http://103.9.213.43</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>123.30.208.19:80</t>
+          <t>103.9.213.43:80</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr"/>
@@ -2817,43 +2717,51 @@
       </c>
       <c r="F90" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>HaNoi Stock Exchange</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>https://123.30.208.19:443</t>
+          <t>http://103.82.192.168</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>123.30.208.19:443</t>
-        </is>
-      </c>
-      <c r="C91" s="6" t="inlineStr"/>
-      <c r="D91" s="6" t="inlineStr"/>
+          <t>103.82.192.168:80</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
       <c r="E91" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Da Nang</t>
         </is>
       </c>
       <c r="F91" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>http://123.31.31.119:49163</t>
+          <t>https://103.82.192.168</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>123.31.31.119:49163</t>
+          <t>103.82.192.168:443</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
@@ -2863,29 +2771,29 @@
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>console-open;T3-open</t>
+          <t>console-open</t>
         </is>
       </c>
       <c r="E92" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Da Nang</t>
         </is>
       </c>
       <c r="F92" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>CLOUDFLY CORPORATION</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>http://123.31.31.125:49163</t>
+          <t>http://103.82.194.3</t>
         </is>
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>123.31.31.125:49163</t>
+          <t>103.82.194.3:80</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
@@ -2895,12 +2803,12 @@
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>console-open;T3-open</t>
+          <t>console-open</t>
         </is>
       </c>
       <c r="E93" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Da Nang</t>
         </is>
       </c>
       <c r="F93" s="6" t="inlineStr">
@@ -2912,16 +2820,20 @@
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>http://123.31.36.60</t>
+          <t>https://103.120.242.145:8081</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>123.31.36.60:80</t>
+          <t>103.120.242.145:8081</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr"/>
-      <c r="D94" s="6" t="inlineStr"/>
+      <c r="D94" s="6" t="inlineStr">
+        <is>
+          <t>console-403</t>
+        </is>
+      </c>
       <c r="E94" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -2929,111 +2841,91 @@
       </c>
       <c r="F94" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>https://123.31.36.60</t>
+          <t>http://103.146.20.88:443</t>
         </is>
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>123.31.36.60:443</t>
+          <t>103.146.20.88:443</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr"/>
       <c r="D95" s="6" t="inlineStr"/>
-      <c r="E95" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="E95" s="6" t="inlineStr"/>
       <c r="F95" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>International Distribution Corporation</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>http://123.31.36.63:8002</t>
+          <t>https://103.150.240.14:443</t>
         </is>
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>123.31.36.63:8002</t>
-        </is>
-      </c>
-      <c r="C96" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D96" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
+          <t>103.150.240.14:443</t>
+        </is>
+      </c>
+      <c r="C96" s="6" t="inlineStr"/>
+      <c r="D96" s="6" t="inlineStr"/>
       <c r="E96" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F96" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>INTELLIGENCE INFORMATION SYSTEM CO, LTD</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>https://124.158.11.115:8443</t>
+          <t>http://103.238.209.174</t>
         </is>
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>124.158.11.115:8443</t>
+          <t>103.238.209.174:80</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr"/>
       <c r="D97" s="6" t="inlineStr"/>
       <c r="E97" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F97" s="6" t="inlineStr">
         <is>
-          <t>CMC Telecom Infrastructure Company</t>
+          <t>VINGROUP JOINT STOCK COMPANY</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>http://160.191.101.129:9001</t>
+          <t>https://103.238.209.174</t>
         </is>
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>160.191.101.129:9001</t>
-        </is>
-      </c>
-      <c r="C98" s="6" t="inlineStr">
-        <is>
-          <t>14.1.2.0.0</t>
-        </is>
-      </c>
-      <c r="D98" s="6" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>103.238.209.174:443</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="inlineStr"/>
+      <c r="D98" s="6" t="inlineStr"/>
       <c r="E98" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3041,51 +2933,43 @@
       </c>
       <c r="F98" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>VINGROUP JOINT STOCK COMPANY</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>http://171.244.38.92:7001</t>
+          <t>https://112.109.89.131</t>
         </is>
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>171.244.38.92:7001</t>
-        </is>
-      </c>
-      <c r="C99" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D99" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>112.109.89.131:443</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="inlineStr"/>
+      <c r="D99" s="6" t="inlineStr"/>
       <c r="E99" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F99" s="6" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>Minh Tu Telecom Limited Company</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>https://183.81.62.19:443</t>
+          <t>http://113.160.181.154:8001</t>
         </is>
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
-          <t>183.81.62.19:443</t>
+          <t>113.160.181.154:8001</t>
         </is>
       </c>
       <c r="C100" s="6" t="inlineStr"/>
@@ -3097,47 +2981,63 @@
       </c>
       <c r="F100" s="6" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>https://202.74.59.145</t>
+          <t>http://113.160.201.159:7001</t>
         </is>
       </c>
       <c r="B101" s="6" t="inlineStr">
         <is>
-          <t>202.74.59.145:443</t>
-        </is>
-      </c>
-      <c r="C101" s="6" t="inlineStr"/>
-      <c r="D101" s="6" t="inlineStr"/>
+          <t>113.160.201.159:7001</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
       <c r="E101" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Thai Binh</t>
         </is>
       </c>
       <c r="F101" s="6" t="inlineStr">
         <is>
-          <t>170 Hai Ba Trung, DaKao Ward, District 1, Hochiminh City</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>http://203.205.28.64:8000</t>
+          <t>http://113.161.43.248:9001</t>
         </is>
       </c>
       <c r="B102" s="6" t="inlineStr">
         <is>
-          <t>203.205.28.64:8000</t>
-        </is>
-      </c>
-      <c r="C102" s="6" t="inlineStr"/>
-      <c r="D102" s="6" t="inlineStr"/>
+          <t>113.161.43.248:9001</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>14.1.2.0.0</t>
+        </is>
+      </c>
+      <c r="D102" s="6" t="inlineStr">
+        <is>
+          <t>T3-open</t>
+        </is>
+      </c>
       <c r="E102" s="6" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
@@ -3145,63 +3045,55 @@
       </c>
       <c r="F102" s="6" t="inlineStr">
         <is>
-          <t>CMC Telecom Infrastructure Company</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>http://210.211.98.79:8080</t>
+          <t>http://113.163.187.3:27001</t>
         </is>
       </c>
       <c r="B103" s="6" t="inlineStr">
         <is>
-          <t>210.211.98.79:8080</t>
+          <t>113.163.187.3:27001</t>
         </is>
       </c>
       <c r="C103" s="6" t="inlineStr">
         <is>
-          <t>14.1.1.0.0</t>
+          <t>10.3.6.0</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>console-open</t>
+          <t>console-open;T3-open</t>
         </is>
       </c>
       <c r="E103" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Phan Rang-Thap Cham</t>
         </is>
       </c>
       <c r="F103" s="6" t="inlineStr">
         <is>
-          <t>CHT Compamy Ltd</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>http://210.211.98.79:8081</t>
+          <t>http://113.185.0.60:8080</t>
         </is>
       </c>
       <c r="B104" s="6" t="inlineStr">
         <is>
-          <t>210.211.98.79:8081</t>
-        </is>
-      </c>
-      <c r="C104" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D104" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>113.185.0.60:8080</t>
+        </is>
+      </c>
+      <c r="C104" s="6" t="inlineStr"/>
+      <c r="D104" s="6" t="inlineStr"/>
       <c r="E104" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3209,25 +3101,29 @@
       </c>
       <c r="F104" s="6" t="inlineStr">
         <is>
-          <t>CHT Compamy Ltd</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>http://210.211.99.108</t>
+          <t>http://117.4.32.40:1111</t>
         </is>
       </c>
       <c r="B105" s="6" t="inlineStr">
         <is>
-          <t>210.211.99.108:80</t>
-        </is>
-      </c>
-      <c r="C105" s="6" t="inlineStr"/>
-      <c r="D105" s="6" t="inlineStr">
-        <is>
-          <t>console-403</t>
+          <t>117.4.32.40:1111</t>
+        </is>
+      </c>
+      <c r="C105" s="6" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
         </is>
       </c>
       <c r="E105" s="6" t="inlineStr">
@@ -3237,25 +3133,29 @@
       </c>
       <c r="F105" s="6" t="inlineStr">
         <is>
-          <t>CHT Compamy Ltd</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>https://210.211.99.108</t>
+          <t>http://117.4.241.247:1112</t>
         </is>
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>210.211.99.108:443</t>
-        </is>
-      </c>
-      <c r="C106" s="6" t="inlineStr"/>
-      <c r="D106" s="6" t="inlineStr">
-        <is>
-          <t>console-403</t>
+          <t>117.4.241.247:1112</t>
+        </is>
+      </c>
+      <c r="C106" s="6" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
         </is>
       </c>
       <c r="E106" s="6" t="inlineStr">
@@ -3265,83 +3165,75 @@
       </c>
       <c r="F106" s="6" t="inlineStr">
         <is>
-          <t>CHT Compamy Ltd</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>http://210.211.99.108:8080</t>
+          <t>https://118.69.32.193:3068</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>210.211.99.108:8080</t>
-        </is>
-      </c>
-      <c r="C107" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D107" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
+          <t>118.69.32.193:3068</t>
+        </is>
+      </c>
+      <c r="C107" s="6" t="inlineStr"/>
+      <c r="D107" s="6" t="inlineStr"/>
       <c r="E107" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Thu Dau Mot</t>
         </is>
       </c>
       <c r="F107" s="6" t="inlineStr">
         <is>
-          <t>CHT Compamy Ltd</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>https://210.211.99.108:9068</t>
+          <t>http://118.69.182.224:9079</t>
         </is>
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>210.211.99.108:9068</t>
+          <t>118.69.182.224:9079</t>
         </is>
       </c>
       <c r="C108" s="6" t="inlineStr">
         <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D108" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D108" s="6" t="inlineStr">
+        <is>
+          <t>T3-open</t>
         </is>
       </c>
       <c r="E108" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Bien Hoa</t>
         </is>
       </c>
       <c r="F108" s="6" t="inlineStr">
         <is>
-          <t>CHT Compamy Ltd</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>https://210.245.45.90</t>
+          <t>http://123.30.208.19:80</t>
         </is>
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>210.245.45.90:443</t>
+          <t>123.30.208.19:80</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr"/>
@@ -3353,12 +3245,760 @@
       </c>
       <c r="F109" s="6" t="inlineStr">
         <is>
+          <t>VNPT Corp</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="5" t="inlineStr">
+        <is>
+          <t>https://123.30.208.19:443</t>
+        </is>
+      </c>
+      <c r="B110" s="6" t="inlineStr">
+        <is>
+          <t>123.30.208.19:443</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="inlineStr"/>
+      <c r="D110" s="6" t="inlineStr"/>
+      <c r="E110" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F110" s="6" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t>http://123.31.31.119:49163</t>
+        </is>
+      </c>
+      <c r="B111" s="6" t="inlineStr">
+        <is>
+          <t>123.31.31.119:49163</t>
+        </is>
+      </c>
+      <c r="C111" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
+      <c r="E111" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F111" s="6" t="inlineStr">
+        <is>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="5" t="inlineStr">
+        <is>
+          <t>http://123.31.31.125:49163</t>
+        </is>
+      </c>
+      <c r="B112" s="6" t="inlineStr">
+        <is>
+          <t>123.31.31.125:49163</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
+      <c r="E112" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F112" s="6" t="inlineStr">
+        <is>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>http://123.31.36.60</t>
+        </is>
+      </c>
+      <c r="B113" s="6" t="inlineStr">
+        <is>
+          <t>123.31.36.60:80</t>
+        </is>
+      </c>
+      <c r="C113" s="6" t="inlineStr"/>
+      <c r="D113" s="6" t="inlineStr"/>
+      <c r="E113" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F113" s="6" t="inlineStr">
+        <is>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="5" t="inlineStr">
+        <is>
+          <t>https://123.31.36.60</t>
+        </is>
+      </c>
+      <c r="B114" s="6" t="inlineStr">
+        <is>
+          <t>123.31.36.60:443</t>
+        </is>
+      </c>
+      <c r="C114" s="6" t="inlineStr"/>
+      <c r="D114" s="6" t="inlineStr"/>
+      <c r="E114" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F114" s="6" t="inlineStr">
+        <is>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="5" t="inlineStr">
+        <is>
+          <t>http://123.31.36.63:8002</t>
+        </is>
+      </c>
+      <c r="B115" s="6" t="inlineStr">
+        <is>
+          <t>123.31.36.63:8002</t>
+        </is>
+      </c>
+      <c r="C115" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
+      <c r="E115" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F115" s="6" t="inlineStr">
+        <is>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="5" t="inlineStr">
+        <is>
+          <t>https://124.158.11.115:8443</t>
+        </is>
+      </c>
+      <c r="B116" s="6" t="inlineStr">
+        <is>
+          <t>124.158.11.115:8443</t>
+        </is>
+      </c>
+      <c r="C116" s="6" t="inlineStr"/>
+      <c r="D116" s="6" t="inlineStr"/>
+      <c r="E116" s="6" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="F116" s="6" t="inlineStr">
+        <is>
+          <t>CMC Telecom Infrastructure Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="5" t="inlineStr">
+        <is>
+          <t>https://144.48.24.66:5620</t>
+        </is>
+      </c>
+      <c r="B117" s="6" t="inlineStr">
+        <is>
+          <t>144.48.24.66:5620</t>
+        </is>
+      </c>
+      <c r="C117" s="6" t="inlineStr"/>
+      <c r="D117" s="6" t="inlineStr"/>
+      <c r="E117" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F117" s="6" t="inlineStr">
+        <is>
+          <t>CMC Telecom Infrastructure Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="5" t="inlineStr">
+        <is>
+          <t>https://144.48.24.66:5650</t>
+        </is>
+      </c>
+      <c r="B118" s="6" t="inlineStr">
+        <is>
+          <t>144.48.24.66:5650</t>
+        </is>
+      </c>
+      <c r="C118" s="6" t="inlineStr"/>
+      <c r="D118" s="6" t="inlineStr"/>
+      <c r="E118" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F118" s="6" t="inlineStr">
+        <is>
+          <t>CMC Telecom Infrastructure Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="inlineStr">
+        <is>
+          <t>https://144.48.24.66:5680</t>
+        </is>
+      </c>
+      <c r="B119" s="6" t="inlineStr">
+        <is>
+          <t>144.48.24.66:5680</t>
+        </is>
+      </c>
+      <c r="C119" s="6" t="inlineStr"/>
+      <c r="D119" s="6" t="inlineStr"/>
+      <c r="E119" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F119" s="6" t="inlineStr">
+        <is>
+          <t>CMC Telecom Infrastructure Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="5" t="inlineStr">
+        <is>
+          <t>https://144.48.24.69:5620</t>
+        </is>
+      </c>
+      <c r="B120" s="6" t="inlineStr">
+        <is>
+          <t>144.48.24.69:5620</t>
+        </is>
+      </c>
+      <c r="C120" s="6" t="inlineStr"/>
+      <c r="D120" s="6" t="inlineStr"/>
+      <c r="E120" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F120" s="6" t="inlineStr">
+        <is>
+          <t>CMC Telecom Infrastructure Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="inlineStr">
+        <is>
+          <t>https://144.48.24.69:5650</t>
+        </is>
+      </c>
+      <c r="B121" s="6" t="inlineStr">
+        <is>
+          <t>144.48.24.69:5650</t>
+        </is>
+      </c>
+      <c r="C121" s="6" t="inlineStr"/>
+      <c r="D121" s="6" t="inlineStr"/>
+      <c r="E121" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F121" s="6" t="inlineStr">
+        <is>
+          <t>CMC Telecom Infrastructure Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="5" t="inlineStr">
+        <is>
+          <t>http://160.191.101.129:9001</t>
+        </is>
+      </c>
+      <c r="B122" s="6" t="inlineStr">
+        <is>
+          <t>160.191.101.129:9001</t>
+        </is>
+      </c>
+      <c r="C122" s="6" t="inlineStr">
+        <is>
+          <t>14.1.2.0.0</t>
+        </is>
+      </c>
+      <c r="D122" s="6" t="inlineStr">
+        <is>
+          <t>T3-open</t>
+        </is>
+      </c>
+      <c r="E122" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F122" s="6" t="inlineStr">
+        <is>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="5" t="inlineStr">
+        <is>
+          <t>http://171.244.38.92:7001</t>
+        </is>
+      </c>
+      <c r="B123" s="6" t="inlineStr">
+        <is>
+          <t>171.244.38.92:7001</t>
+        </is>
+      </c>
+      <c r="C123" s="6" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
+      <c r="E123" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F123" s="6" t="inlineStr">
+        <is>
+          <t>Viettel Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="5" t="inlineStr">
+        <is>
+          <t>http://171.254.93.47:9505</t>
+        </is>
+      </c>
+      <c r="B124" s="6" t="inlineStr">
+        <is>
+          <t>171.254.93.47:9505</t>
+        </is>
+      </c>
+      <c r="C124" s="6" t="inlineStr"/>
+      <c r="D124" s="6" t="inlineStr"/>
+      <c r="E124" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F124" s="6" t="inlineStr">
+        <is>
+          <t>Viettel Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>https://183.81.62.19:443</t>
+        </is>
+      </c>
+      <c r="B125" s="6" t="inlineStr">
+        <is>
+          <t>183.81.62.19:443</t>
+        </is>
+      </c>
+      <c r="C125" s="6" t="inlineStr"/>
+      <c r="D125" s="6" t="inlineStr"/>
+      <c r="E125" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F125" s="6" t="inlineStr">
+        <is>
           <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" s="5" t="inlineStr">
+        <is>
+          <t>https://202.74.59.145</t>
+        </is>
+      </c>
+      <c r="B126" s="6" t="inlineStr">
+        <is>
+          <t>202.74.59.145:443</t>
+        </is>
+      </c>
+      <c r="C126" s="6" t="inlineStr"/>
+      <c r="D126" s="6" t="inlineStr"/>
+      <c r="E126" s="6" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="F126" s="6" t="inlineStr">
+        <is>
+          <t>170 Hai Ba Trung, DaKao Ward, District 1, Hochiminh City</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>https://203.189.31.24</t>
+        </is>
+      </c>
+      <c r="B127" s="6" t="inlineStr">
+        <is>
+          <t>203.189.31.24:443</t>
+        </is>
+      </c>
+      <c r="C127" s="6" t="inlineStr"/>
+      <c r="D127" s="6" t="inlineStr"/>
+      <c r="E127" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F127" s="6" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="5" t="inlineStr">
+        <is>
+          <t>http://203.205.28.64:8000</t>
+        </is>
+      </c>
+      <c r="B128" s="6" t="inlineStr">
+        <is>
+          <t>203.205.28.64:8000</t>
+        </is>
+      </c>
+      <c r="C128" s="6" t="inlineStr"/>
+      <c r="D128" s="6" t="inlineStr"/>
+      <c r="E128" s="6" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="F128" s="6" t="inlineStr">
+        <is>
+          <t>CMC Telecom Infrastructure Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="inlineStr">
+        <is>
+          <t>https://203.205.57.229:443</t>
+        </is>
+      </c>
+      <c r="B129" s="6" t="inlineStr">
+        <is>
+          <t>203.205.57.229:443</t>
+        </is>
+      </c>
+      <c r="C129" s="6" t="inlineStr"/>
+      <c r="D129" s="6" t="inlineStr"/>
+      <c r="E129" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F129" s="6" t="inlineStr">
+        <is>
+          <t>CMC Telecom Infrastructure Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="5" t="inlineStr">
+        <is>
+          <t>http://210.211.98.79:8080</t>
+        </is>
+      </c>
+      <c r="B130" s="6" t="inlineStr">
+        <is>
+          <t>210.211.98.79:8080</t>
+        </is>
+      </c>
+      <c r="C130" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D130" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
+      <c r="E130" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F130" s="6" t="inlineStr">
+        <is>
+          <t>CHT Compamy Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="inlineStr">
+        <is>
+          <t>http://210.211.98.79:8081</t>
+        </is>
+      </c>
+      <c r="B131" s="6" t="inlineStr">
+        <is>
+          <t>210.211.98.79:8081</t>
+        </is>
+      </c>
+      <c r="C131" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D131" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
+      <c r="E131" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F131" s="6" t="inlineStr">
+        <is>
+          <t>CHT Compamy Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="5" t="inlineStr">
+        <is>
+          <t>https://210.211.99.108</t>
+        </is>
+      </c>
+      <c r="B132" s="6" t="inlineStr">
+        <is>
+          <t>210.211.99.108:443</t>
+        </is>
+      </c>
+      <c r="C132" s="6" t="inlineStr"/>
+      <c r="D132" s="6" t="inlineStr">
+        <is>
+          <t>console-403</t>
+        </is>
+      </c>
+      <c r="E132" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F132" s="6" t="inlineStr">
+        <is>
+          <t>CHT Compamy Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="5" t="inlineStr">
+        <is>
+          <t>http://210.211.99.108:7023</t>
+        </is>
+      </c>
+      <c r="B133" s="6" t="inlineStr">
+        <is>
+          <t>210.211.99.108:7023</t>
+        </is>
+      </c>
+      <c r="C133" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D133" s="6" t="inlineStr">
+        <is>
+          <t>console-403;T3-open</t>
+        </is>
+      </c>
+      <c r="E133" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F133" s="6" t="inlineStr">
+        <is>
+          <t>CHT Compamy Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="5" t="inlineStr">
+        <is>
+          <t>https://210.211.99.108:9023</t>
+        </is>
+      </c>
+      <c r="B134" s="6" t="inlineStr">
+        <is>
+          <t>210.211.99.108:9023</t>
+        </is>
+      </c>
+      <c r="C134" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D134" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
+      <c r="E134" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F134" s="6" t="inlineStr">
+        <is>
+          <t>CHT Compamy Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>https://210.211.99.108:9068</t>
+        </is>
+      </c>
+      <c r="B135" s="6" t="inlineStr">
+        <is>
+          <t>210.211.99.108:9068</t>
+        </is>
+      </c>
+      <c r="C135" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D135" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
+      <c r="E135" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F135" s="6" t="inlineStr">
+        <is>
+          <t>CHT Compamy Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="5" t="inlineStr">
+        <is>
+          <t>https://210.245.45.90</t>
+        </is>
+      </c>
+      <c r="B136" s="6" t="inlineStr">
+        <is>
+          <t>210.245.45.90:443</t>
+        </is>
+      </c>
+      <c r="C136" s="6" t="inlineStr"/>
+      <c r="D136" s="6" t="inlineStr"/>
+      <c r="E136" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F136" s="6" t="inlineStr">
+        <is>
+          <t>FPT Telecom Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>https://210.245.119.65</t>
+        </is>
+      </c>
+      <c r="B137" s="6" t="inlineStr">
+        <is>
+          <t>210.245.119.65:443</t>
+        </is>
+      </c>
+      <c r="C137" s="6" t="inlineStr"/>
+      <c r="D137" s="6" t="inlineStr"/>
+      <c r="E137" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F137" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F109"/>
+  <autoFilter ref="A1:F137"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
@@ -3468,6 +4108,34 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A107" r:id="rId106"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A108" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A137" r:id="rId136"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
vault backup: 2026-10-09 12:11:13
</commit_message>
<xml_diff>
--- a/WLS-VN-live.xlsx
+++ b/WLS-VN-live.xlsx
@@ -10,7 +10,7 @@
     <sheet name="WLS VN (live)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WLS VN (live)'!$A$1:$F$137</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WLS VN (live)'!$A$1:$F$135</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F137"/>
+  <dimension ref="A1:F135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1692,12 +1692,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>http://trienlamso.ictquangtri.vn</t>
+          <t>http://capcaohcm.toaan.gov.vn</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>117.122.125.107:80</t>
+          <t>123.30.24.180:80</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr"/>
@@ -1709,19 +1709,19 @@
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Internet Network Information Center</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>https://euroeximbank.com.vn</t>
+          <t>https://mla.toaan.gov.vn</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>117.122.125.107:443</t>
+          <t>123.30.24.180:443</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr"/>
@@ -1733,19 +1733,19 @@
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Internet Network Information Center</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>http://capcaohcm.toaan.gov.vn</t>
+          <t>https://cskh.temxacthuc.vn:8081</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>123.30.24.180:80</t>
+          <t>123.30.208.19:8081</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr"/>
@@ -1764,12 +1764,12 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>https://mla.toaan.gov.vn</t>
+          <t>http://www.topteen.vn</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>123.30.24.180:443</t>
+          <t>123.30.208.25:80</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr"/>
@@ -1788,12 +1788,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>https://cskh.temxacthuc.vn:8081</t>
+          <t>http://gmobi.vn</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>123.30.208.19:8081</t>
+          <t>123.31.31.126:80</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr"/>
@@ -1805,19 +1805,19 @@
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>http://www.topteen.vn</t>
+          <t>http://cskh.temdientu.vn</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>123.30.208.25:80</t>
+          <t>123.31.41.93:80</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr"/>
@@ -1829,19 +1829,19 @@
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>http://gmobi.vn</t>
+          <t>http://csdlgiaquocgia.mof.gov.vn</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>123.31.31.126:80</t>
+          <t>182.236.113.46:80</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr"/>
@@ -1853,19 +1853,19 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>Department of Information Technology and Digital Transformation - Ministry of Finance</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>http://cskh.temdientu.vn</t>
+          <t>https://csdlgiaquocgia.mof.gov.vn</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>123.31.41.93:80</t>
+          <t>182.236.113.46:443</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr"/>
@@ -1877,115 +1877,115 @@
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>Department of Information Technology and Digital Transformation - Ministry of Finance</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>http://csdlgiaquocgia.mof.gov.vn</t>
+          <t>http://thongbaotenmien.vn</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>182.236.113.46:80</t>
+          <t>203.119.73.12:80</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr"/>
       <c r="D57" s="3" t="inlineStr"/>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>Department of Information Technology and Digital Transformation - Ministry of Finance</t>
+          <t>Vietnam Internet network information center (VNNIC)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>https://csdlgiaquocgia.mof.gov.vn</t>
+          <t>https://thongbaotenmien.vn</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>182.236.113.46:443</t>
+          <t>203.119.73.12:443</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr"/>
       <c r="D58" s="3" t="inlineStr"/>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Department of Information Technology and Digital Transformation - Ministry of Finance</t>
+          <t>Vietnam Internet network information center (VNNIC)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>http://thongbaotenmien.vn</t>
+          <t>http://qlahs.vksndtc.gov.vn</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>203.119.73.12:80</t>
+          <t>203.162.255.5:80</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr"/>
       <c r="D59" s="3" t="inlineStr"/>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Internet network information center (VNNIC)</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>https://thongbaotenmien.vn</t>
+          <t>http://chuyentien.vietinbank.vn</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>203.119.73.12:443</t>
+          <t>203.189.28.86:80</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr"/>
       <c r="D60" s="3" t="inlineStr"/>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Internet network information center (VNNIC)</t>
+          <t>VIETINBANK</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>http://qlahs.vksndtc.gov.vn</t>
+          <t>http://sso.vietinbank.vn</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>203.162.255.5:80</t>
+          <t>203.189.29.33:80</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr"/>
@@ -1997,19 +1997,19 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>VIETINBANK-VN</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>http://chuyentien.vietinbank.vn</t>
+          <t>https://sso.vietinbank.vn</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>203.189.28.86:80</t>
+          <t>203.189.29.33:443</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr"/>
@@ -2021,74 +2021,82 @@
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>VIETINBANK</t>
+          <t>VIETINBANK-VN</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>http://sso.vietinbank.vn</t>
+          <t>http://htttsv.hoasen.edu.vn</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>203.189.29.33:80</t>
+          <t>203.205.57.225:80</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr"/>
       <c r="D63" s="3" t="inlineStr"/>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>VIETINBANK-VN</t>
+          <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>https://sso.vietinbank.vn</t>
+          <t>https://htttsv.hoasen.edu.vn</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>203.189.29.33:443</t>
+          <t>203.205.57.225:443</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr"/>
       <c r="D64" s="3" t="inlineStr"/>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>VIETINBANK-VN</t>
+          <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>http://htttsv.hoasen.edu.vn</t>
+          <t>http://erpbk.hoasen.edu.vn</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>203.205.57.225:80</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="inlineStr"/>
-      <c r="D65" s="3" t="inlineStr"/>
+          <t>203.205.57.226:80</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>10.3.4.0</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
@@ -2100,48 +2108,40 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>https://htttsv.hoasen.edu.vn</t>
+          <t>http://cms.mebongda.net</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>203.205.57.225:443</t>
+          <t>210.211.99.108:80</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr"/>
       <c r="D66" s="3" t="inlineStr"/>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>CMC Telecom Infrastructure Company</t>
+          <t>CHT Compamy Ltd</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>http://erpbk.hoasen.edu.vn</t>
+          <t>http://static.ketquasieutoc.com:8080</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>203.205.57.226:80</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="inlineStr">
-        <is>
-          <t>10.3.4.0</t>
-        </is>
-      </c>
-      <c r="D67" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
+          <t>210.211.99.108:8080</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr"/>
+      <c r="D67" s="3" t="inlineStr"/>
       <c r="E67" s="3" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -2149,19 +2149,19 @@
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>CMC Telecom Infrastructure Company</t>
+          <t>CHT Compamy Ltd</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>http://cms.mebongda.net</t>
+          <t>http://mobilaw.vn</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>210.211.99.108:80</t>
+          <t>210.211.99.130:80</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr"/>
@@ -2171,21 +2171,17 @@
           <t>Hanoi</t>
         </is>
       </c>
-      <c r="F68" s="3" t="inlineStr">
-        <is>
-          <t>CHT Compamy Ltd</t>
-        </is>
-      </c>
+      <c r="F68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>http://static.ketquasieutoc.com:8080</t>
+          <t>http://m.xosothongminh.vn</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>210.211.99.108:8080</t>
+          <t>210.211.99.133:80</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr"/>
@@ -2195,21 +2191,17 @@
           <t>Hanoi</t>
         </is>
       </c>
-      <c r="F69" s="3" t="inlineStr">
-        <is>
-          <t>CHT Compamy Ltd</t>
-        </is>
-      </c>
+      <c r="F69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>http://mobilaw.vn</t>
+          <t>http://rvt.kenhnhac.vn</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>210.211.99.130:80</t>
+          <t>210.211.99.174:80</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr"/>
@@ -2219,17 +2211,21 @@
           <t>Hanoi</t>
         </is>
       </c>
-      <c r="F70" s="3" t="inlineStr"/>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>CHT Compamy Ltd</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>http://m.xosothongminh.vn</t>
+          <t>http://dvc-kbnn.fintechviet.vn</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>210.211.99.133:80</t>
+          <t>222.252.98.4:80</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr"/>
@@ -2239,51 +2235,63 @@
           <t>Hanoi</t>
         </is>
       </c>
-      <c r="F71" s="3" t="inlineStr"/>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
+        </is>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>http://rvt.kenhnhac.vn</t>
-        </is>
-      </c>
-      <c r="B72" s="3" t="inlineStr">
-        <is>
-          <t>210.211.99.174:80</t>
-        </is>
-      </c>
-      <c r="C72" s="3" t="inlineStr"/>
-      <c r="D72" s="3" t="inlineStr"/>
-      <c r="E72" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F72" s="3" t="inlineStr">
-        <is>
-          <t>CHT Compamy Ltd</t>
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>http://14.225.11.33:9001</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>14.225.11.33:9001</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>T3-open</t>
+        </is>
+      </c>
+      <c r="E72" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="inlineStr">
+        <is>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>http://dvc-kbnn.fintechviet.vn</t>
-        </is>
-      </c>
-      <c r="B73" s="3" t="inlineStr">
-        <is>
-          <t>222.252.98.4:80</t>
-        </is>
-      </c>
-      <c r="C73" s="3" t="inlineStr"/>
-      <c r="D73" s="3" t="inlineStr"/>
-      <c r="E73" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F73" s="3" t="inlineStr">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>http://14.238.41.12:80</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>14.238.41.12:80</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr"/>
+      <c r="D73" s="6" t="inlineStr"/>
+      <c r="E73" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
         </is>
@@ -2292,51 +2300,43 @@
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>http://14.225.11.33:9001</t>
+          <t>https://14.238.93.114:9184</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>14.225.11.33:9001</t>
-        </is>
-      </c>
-      <c r="C74" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D74" s="6" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>14.238.93.114:9184</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr"/>
+      <c r="D74" s="6" t="inlineStr"/>
       <c r="E74" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>http://14.238.41.12:80</t>
+          <t>http://14.241.253.96:8081</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>14.238.41.12:80</t>
+          <t>14.241.253.96:8081</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr"/>
       <c r="D75" s="6" t="inlineStr"/>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F75" s="6" t="inlineStr">
@@ -2348,12 +2348,12 @@
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>https://14.238.93.114:9184</t>
+          <t>http://14.241.253.96:8082</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>14.238.93.114:9184</t>
+          <t>14.241.253.96:8082</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr"/>
@@ -2372,19 +2372,19 @@
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>http://14.241.253.96:8081</t>
+          <t>https://14.248.84.7:443</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>14.241.253.96:8081</t>
+          <t>14.248.84.7:443</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr"/>
       <c r="D77" s="6" t="inlineStr"/>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F77" s="6" t="inlineStr">
@@ -2396,132 +2396,140 @@
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>http://14.241.253.96:8082</t>
+          <t>http://27.72.123.124:8001</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>14.241.253.96:8082</t>
+          <t>27.72.123.124:8001</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr"/>
       <c r="D78" s="6" t="inlineStr"/>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Sa Pa</t>
         </is>
       </c>
       <c r="F78" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>https://14.248.84.7:443</t>
+          <t>http://27.72.123.124:8003</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>14.248.84.7:443</t>
+          <t>27.72.123.124:8003</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr"/>
       <c r="D79" s="6" t="inlineStr"/>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ha Long</t>
         </is>
       </c>
       <c r="F79" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>http://27.72.123.124:8001</t>
+          <t>https://42.115.41.27:443</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>27.72.123.124:8001</t>
+          <t>42.115.41.27:443</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr"/>
       <c r="D80" s="6" t="inlineStr"/>
       <c r="E80" s="6" t="inlineStr">
         <is>
-          <t>Sa Pa</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F80" s="6" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>http://27.72.123.124:8003</t>
+          <t>http://42.118.60.193:7001</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>27.72.123.124:8003</t>
-        </is>
-      </c>
-      <c r="C81" s="6" t="inlineStr"/>
-      <c r="D81" s="6" t="inlineStr"/>
+          <t>42.118.60.193:7001</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
       <c r="E81" s="6" t="inlineStr">
         <is>
-          <t>Ha Long</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F81" s="6" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>https://42.115.41.27:443</t>
+          <t>https://45.120.230.45</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>42.115.41.27:443</t>
+          <t>45.120.230.45:443</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr"/>
       <c r="D82" s="6" t="inlineStr"/>
       <c r="E82" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F82" s="6" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>Creative Communication Vietnam Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>http://42.118.60.193:7001</t>
+          <t>http://49.213.88.170:7001</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>42.118.60.193:7001</t>
+          <t>49.213.88.170:7001</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
@@ -2536,24 +2544,24 @@
       </c>
       <c r="E83" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F83" s="6" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>VNG Corporation</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>https://45.120.230.45</t>
+          <t>https://103.3.252.106:7002</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>45.120.230.45:443</t>
+          <t>103.3.252.106:7002</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr"/>
@@ -2565,51 +2573,43 @@
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>http://49.213.88.170:7001</t>
+          <t>https://103.3.252.107:7002</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>49.213.88.170:7001</t>
-        </is>
-      </c>
-      <c r="C85" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D85" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>103.3.252.107:7002</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr"/>
+      <c r="D85" s="6" t="inlineStr"/>
       <c r="E85" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F85" s="6" t="inlineStr">
         <is>
-          <t>VNG Corporation</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>https://103.3.252.106:7002</t>
+          <t>http://103.3.252.109:80</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>103.3.252.106:7002</t>
+          <t>103.3.252.109:80</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr"/>
@@ -2628,12 +2628,12 @@
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>https://103.3.252.107:7002</t>
+          <t>http://103.3.252.133</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>103.3.252.107:7002</t>
+          <t>103.3.252.133:80</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr"/>
@@ -2652,12 +2652,12 @@
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>http://103.3.252.109:80</t>
+          <t>http://103.9.213.43</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>103.3.252.109:80</t>
+          <t>103.9.213.43:80</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr"/>
@@ -2669,67 +2669,83 @@
       </c>
       <c r="F88" s="6" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>HaNoi Stock Exchange</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>http://103.3.252.133</t>
+          <t>http://103.82.192.168</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>103.3.252.133:80</t>
-        </is>
-      </c>
-      <c r="C89" s="6" t="inlineStr"/>
-      <c r="D89" s="6" t="inlineStr"/>
+          <t>103.82.192.168:80</t>
+        </is>
+      </c>
+      <c r="C89" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Da Nang</t>
         </is>
       </c>
       <c r="F89" s="6" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>http://103.9.213.43</t>
+          <t>https://103.82.192.168</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>103.9.213.43:80</t>
-        </is>
-      </c>
-      <c r="C90" s="6" t="inlineStr"/>
-      <c r="D90" s="6" t="inlineStr"/>
+          <t>103.82.192.168:443</t>
+        </is>
+      </c>
+      <c r="C90" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
       <c r="E90" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Da Nang</t>
         </is>
       </c>
       <c r="F90" s="6" t="inlineStr">
         <is>
-          <t>HaNoi Stock Exchange</t>
+          <t>CLOUDFLY CORPORATION</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>http://103.82.192.168</t>
+          <t>http://103.82.194.3</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>103.82.192.168:80</t>
+          <t>103.82.194.3:80</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
@@ -2756,172 +2772,156 @@
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>https://103.82.192.168</t>
+          <t>https://103.120.242.145:8081</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>103.82.192.168:443</t>
-        </is>
-      </c>
-      <c r="C92" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D92" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
+          <t>103.120.242.145:8081</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr"/>
+      <c r="D92" s="6" t="inlineStr">
+        <is>
+          <t>console-403</t>
         </is>
       </c>
       <c r="E92" s="6" t="inlineStr">
         <is>
-          <t>Da Nang</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F92" s="6" t="inlineStr">
         <is>
-          <t>CLOUDFLY CORPORATION</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>http://103.82.194.3</t>
+          <t>http://103.146.20.88:443</t>
         </is>
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>103.82.194.3:80</t>
-        </is>
-      </c>
-      <c r="C93" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D93" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
-      <c r="E93" s="6" t="inlineStr">
-        <is>
-          <t>Da Nang</t>
-        </is>
-      </c>
+          <t>103.146.20.88:443</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="inlineStr"/>
+      <c r="D93" s="6" t="inlineStr"/>
+      <c r="E93" s="6" t="inlineStr"/>
       <c r="F93" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>International Distribution Corporation</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>https://103.120.242.145:8081</t>
+          <t>https://103.150.240.14:443</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>103.120.242.145:8081</t>
+          <t>103.150.240.14:443</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr"/>
-      <c r="D94" s="6" t="inlineStr">
-        <is>
-          <t>console-403</t>
-        </is>
-      </c>
+      <c r="D94" s="6" t="inlineStr"/>
       <c r="E94" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F94" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>INTELLIGENCE INFORMATION SYSTEM CO, LTD</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>http://103.146.20.88:443</t>
+          <t>http://103.238.209.174</t>
         </is>
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>103.146.20.88:443</t>
+          <t>103.238.209.174:80</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr"/>
       <c r="D95" s="6" t="inlineStr"/>
-      <c r="E95" s="6" t="inlineStr"/>
+      <c r="E95" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
       <c r="F95" s="6" t="inlineStr">
         <is>
-          <t>International Distribution Corporation</t>
+          <t>VINGROUP JOINT STOCK COMPANY</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>https://103.150.240.14:443</t>
+          <t>https://103.238.209.174</t>
         </is>
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>103.150.240.14:443</t>
+          <t>103.238.209.174:443</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr"/>
       <c r="D96" s="6" t="inlineStr"/>
       <c r="E96" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F96" s="6" t="inlineStr">
         <is>
-          <t>INTELLIGENCE INFORMATION SYSTEM CO, LTD</t>
+          <t>VINGROUP JOINT STOCK COMPANY</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>http://103.238.209.174</t>
+          <t>https://112.109.89.131</t>
         </is>
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>103.238.209.174:80</t>
+          <t>112.109.89.131:443</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr"/>
       <c r="D97" s="6" t="inlineStr"/>
       <c r="E97" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F97" s="6" t="inlineStr">
         <is>
-          <t>VINGROUP JOINT STOCK COMPANY</t>
+          <t>Minh Tu Telecom Limited Company</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>https://103.238.209.174</t>
+          <t>http://113.160.181.154:8001</t>
         </is>
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>103.238.209.174:443</t>
+          <t>113.160.181.154:8001</t>
         </is>
       </c>
       <c r="C98" s="6" t="inlineStr"/>
@@ -2933,50 +2933,66 @@
       </c>
       <c r="F98" s="6" t="inlineStr">
         <is>
-          <t>VINGROUP JOINT STOCK COMPANY</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>https://112.109.89.131</t>
+          <t>http://113.160.201.159:7001</t>
         </is>
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>112.109.89.131:443</t>
-        </is>
-      </c>
-      <c r="C99" s="6" t="inlineStr"/>
-      <c r="D99" s="6" t="inlineStr"/>
+          <t>113.160.201.159:7001</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
       <c r="E99" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Thai Binh</t>
         </is>
       </c>
       <c r="F99" s="6" t="inlineStr">
         <is>
-          <t>Minh Tu Telecom Limited Company</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>http://113.160.181.154:8001</t>
+          <t>http://113.161.43.248:9001</t>
         </is>
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
-          <t>113.160.181.154:8001</t>
-        </is>
-      </c>
-      <c r="C100" s="6" t="inlineStr"/>
-      <c r="D100" s="6" t="inlineStr"/>
+          <t>113.161.43.248:9001</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="inlineStr">
+        <is>
+          <t>14.1.2.0.0</t>
+        </is>
+      </c>
+      <c r="D100" s="6" t="inlineStr">
+        <is>
+          <t>T3-open</t>
+        </is>
+      </c>
       <c r="E100" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F100" s="6" t="inlineStr">
@@ -2988,12 +3004,12 @@
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>http://113.160.201.159:7001</t>
+          <t>http://113.163.187.3:27001</t>
         </is>
       </c>
       <c r="B101" s="6" t="inlineStr">
         <is>
-          <t>113.160.201.159:7001</t>
+          <t>113.163.187.3:27001</t>
         </is>
       </c>
       <c r="C101" s="6" t="inlineStr">
@@ -3008,7 +3024,7 @@
       </c>
       <c r="E101" s="6" t="inlineStr">
         <is>
-          <t>Thai Binh</t>
+          <t>Phan Rang-Thap Cham</t>
         </is>
       </c>
       <c r="F101" s="6" t="inlineStr">
@@ -3020,27 +3036,19 @@
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>http://113.161.43.248:9001</t>
+          <t>http://113.185.0.60:8080</t>
         </is>
       </c>
       <c r="B102" s="6" t="inlineStr">
         <is>
-          <t>113.161.43.248:9001</t>
-        </is>
-      </c>
-      <c r="C102" s="6" t="inlineStr">
-        <is>
-          <t>14.1.2.0.0</t>
-        </is>
-      </c>
-      <c r="D102" s="6" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>113.185.0.60:8080</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="inlineStr"/>
+      <c r="D102" s="6" t="inlineStr"/>
       <c r="E102" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F102" s="6" t="inlineStr">
@@ -3052,12 +3060,12 @@
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>http://113.163.187.3:27001</t>
+          <t>http://117.4.32.40:1111</t>
         </is>
       </c>
       <c r="B103" s="6" t="inlineStr">
         <is>
-          <t>113.163.187.3:27001</t>
+          <t>117.4.32.40:1111</t>
         </is>
       </c>
       <c r="C103" s="6" t="inlineStr">
@@ -3072,28 +3080,36 @@
       </c>
       <c r="E103" s="6" t="inlineStr">
         <is>
-          <t>Phan Rang-Thap Cham</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F103" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>http://113.185.0.60:8080</t>
+          <t>http://117.4.241.247:1112</t>
         </is>
       </c>
       <c r="B104" s="6" t="inlineStr">
         <is>
-          <t>113.185.0.60:8080</t>
-        </is>
-      </c>
-      <c r="C104" s="6" t="inlineStr"/>
-      <c r="D104" s="6" t="inlineStr"/>
+          <t>117.4.241.247:1112</t>
+        </is>
+      </c>
+      <c r="C104" s="6" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
       <c r="E104" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3101,51 +3117,43 @@
       </c>
       <c r="F104" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>http://117.4.32.40:1111</t>
+          <t>https://118.69.32.193:3068</t>
         </is>
       </c>
       <c r="B105" s="6" t="inlineStr">
         <is>
-          <t>117.4.32.40:1111</t>
-        </is>
-      </c>
-      <c r="C105" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D105" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>118.69.32.193:3068</t>
+        </is>
+      </c>
+      <c r="C105" s="6" t="inlineStr"/>
+      <c r="D105" s="6" t="inlineStr"/>
       <c r="E105" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Thu Dau Mot</t>
         </is>
       </c>
       <c r="F105" s="6" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>http://117.4.241.247:1112</t>
+          <t>http://118.69.182.224:9079</t>
         </is>
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>117.4.241.247:1112</t>
+          <t>118.69.182.224:9079</t>
         </is>
       </c>
       <c r="C106" s="6" t="inlineStr">
@@ -3153,91 +3161,91 @@
           <t>10.3.6.0</t>
         </is>
       </c>
-      <c r="D106" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
+      <c r="D106" s="6" t="inlineStr">
+        <is>
+          <t>T3-open</t>
         </is>
       </c>
       <c r="E106" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Bien Hoa</t>
         </is>
       </c>
       <c r="F106" s="6" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>https://118.69.32.193:3068</t>
+          <t>http://123.30.208.19:80</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>118.69.32.193:3068</t>
+          <t>123.30.208.19:80</t>
         </is>
       </c>
       <c r="C107" s="6" t="inlineStr"/>
       <c r="D107" s="6" t="inlineStr"/>
       <c r="E107" s="6" t="inlineStr">
         <is>
-          <t>Thu Dau Mot</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F107" s="6" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>http://118.69.182.224:9079</t>
+          <t>https://123.30.208.19:443</t>
         </is>
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>118.69.182.224:9079</t>
-        </is>
-      </c>
-      <c r="C108" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D108" s="6" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>123.30.208.19:443</t>
+        </is>
+      </c>
+      <c r="C108" s="6" t="inlineStr"/>
+      <c r="D108" s="6" t="inlineStr"/>
       <c r="E108" s="6" t="inlineStr">
         <is>
-          <t>Bien Hoa</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F108" s="6" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>http://123.30.208.19:80</t>
+          <t>http://123.31.31.119:49163</t>
         </is>
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>123.30.208.19:80</t>
-        </is>
-      </c>
-      <c r="C109" s="6" t="inlineStr"/>
-      <c r="D109" s="6" t="inlineStr"/>
+          <t>123.31.31.119:49163</t>
+        </is>
+      </c>
+      <c r="C109" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
       <c r="E109" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3245,23 +3253,31 @@
       </c>
       <c r="F109" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>https://123.30.208.19:443</t>
+          <t>http://123.31.31.125:49163</t>
         </is>
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>123.30.208.19:443</t>
-        </is>
-      </c>
-      <c r="C110" s="6" t="inlineStr"/>
-      <c r="D110" s="6" t="inlineStr"/>
+          <t>123.31.31.125:49163</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
       <c r="E110" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3269,31 +3285,23 @@
       </c>
       <c r="F110" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>http://123.31.31.119:49163</t>
+          <t>http://123.31.36.60</t>
         </is>
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>123.31.31.119:49163</t>
-        </is>
-      </c>
-      <c r="C111" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D111" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>123.31.36.60:80</t>
+        </is>
+      </c>
+      <c r="C111" s="6" t="inlineStr"/>
+      <c r="D111" s="6" t="inlineStr"/>
       <c r="E111" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3308,24 +3316,16 @@
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
         <is>
-          <t>http://123.31.31.125:49163</t>
+          <t>https://123.31.36.60</t>
         </is>
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>123.31.31.125:49163</t>
-        </is>
-      </c>
-      <c r="C112" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D112" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>123.31.36.60:443</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="inlineStr"/>
+      <c r="D112" s="6" t="inlineStr"/>
       <c r="E112" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3340,16 +3340,24 @@
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>http://123.31.36.60</t>
+          <t>http://123.31.36.63:8002</t>
         </is>
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>123.31.36.60:80</t>
-        </is>
-      </c>
-      <c r="C113" s="6" t="inlineStr"/>
-      <c r="D113" s="6" t="inlineStr"/>
+          <t>123.31.36.63:8002</t>
+        </is>
+      </c>
+      <c r="C113" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D113" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
       <c r="E113" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3364,48 +3372,40 @@
     <row r="114">
       <c r="A114" s="5" t="inlineStr">
         <is>
-          <t>https://123.31.36.60</t>
+          <t>https://124.158.11.115:8443</t>
         </is>
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>123.31.36.60:443</t>
+          <t>124.158.11.115:8443</t>
         </is>
       </c>
       <c r="C114" s="6" t="inlineStr"/>
       <c r="D114" s="6" t="inlineStr"/>
       <c r="E114" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F114" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>http://123.31.36.63:8002</t>
+          <t>https://144.48.24.66:5620</t>
         </is>
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>123.31.36.63:8002</t>
-        </is>
-      </c>
-      <c r="C115" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D115" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>144.48.24.66:5620</t>
+        </is>
+      </c>
+      <c r="C115" s="6" t="inlineStr"/>
+      <c r="D115" s="6" t="inlineStr"/>
       <c r="E115" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3413,26 +3413,26 @@
       </c>
       <c r="F115" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>https://124.158.11.115:8443</t>
+          <t>https://144.48.24.66:5650</t>
         </is>
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
-          <t>124.158.11.115:8443</t>
+          <t>144.48.24.66:5650</t>
         </is>
       </c>
       <c r="C116" s="6" t="inlineStr"/>
       <c r="D116" s="6" t="inlineStr"/>
       <c r="E116" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F116" s="6" t="inlineStr">
@@ -3444,12 +3444,12 @@
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>https://144.48.24.66:5620</t>
+          <t>https://144.48.24.66:5680</t>
         </is>
       </c>
       <c r="B117" s="6" t="inlineStr">
         <is>
-          <t>144.48.24.66:5620</t>
+          <t>144.48.24.66:5680</t>
         </is>
       </c>
       <c r="C117" s="6" t="inlineStr"/>
@@ -3468,12 +3468,12 @@
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
         <is>
-          <t>https://144.48.24.66:5650</t>
+          <t>https://144.48.24.69:5620</t>
         </is>
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>144.48.24.66:5650</t>
+          <t>144.48.24.69:5620</t>
         </is>
       </c>
       <c r="C118" s="6" t="inlineStr"/>
@@ -3492,12 +3492,12 @@
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>https://144.48.24.66:5680</t>
+          <t>https://144.48.24.69:5650</t>
         </is>
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>144.48.24.66:5680</t>
+          <t>144.48.24.69:5650</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr"/>
@@ -3516,16 +3516,24 @@
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
-          <t>https://144.48.24.69:5620</t>
+          <t>http://160.191.101.129:9001</t>
         </is>
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>144.48.24.69:5620</t>
-        </is>
-      </c>
-      <c r="C120" s="6" t="inlineStr"/>
-      <c r="D120" s="6" t="inlineStr"/>
+          <t>160.191.101.129:9001</t>
+        </is>
+      </c>
+      <c r="C120" s="6" t="inlineStr">
+        <is>
+          <t>14.1.2.0.0</t>
+        </is>
+      </c>
+      <c r="D120" s="6" t="inlineStr">
+        <is>
+          <t>T3-open</t>
+        </is>
+      </c>
       <c r="E120" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3533,23 +3541,31 @@
       </c>
       <c r="F120" s="6" t="inlineStr">
         <is>
-          <t>CMC Telecom Infrastructure Company</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>https://144.48.24.69:5650</t>
+          <t>http://171.244.38.92:7001</t>
         </is>
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>144.48.24.69:5650</t>
-        </is>
-      </c>
-      <c r="C121" s="6" t="inlineStr"/>
-      <c r="D121" s="6" t="inlineStr"/>
+          <t>171.244.38.92:7001</t>
+        </is>
+      </c>
+      <c r="C121" s="6" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D121" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
       <c r="E121" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3557,31 +3573,23 @@
       </c>
       <c r="F121" s="6" t="inlineStr">
         <is>
-          <t>CMC Telecom Infrastructure Company</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
         <is>
-          <t>http://160.191.101.129:9001</t>
+          <t>http://171.254.93.47:9505</t>
         </is>
       </c>
       <c r="B122" s="6" t="inlineStr">
         <is>
-          <t>160.191.101.129:9001</t>
-        </is>
-      </c>
-      <c r="C122" s="6" t="inlineStr">
-        <is>
-          <t>14.1.2.0.0</t>
-        </is>
-      </c>
-      <c r="D122" s="6" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>171.254.93.47:9505</t>
+        </is>
+      </c>
+      <c r="C122" s="6" t="inlineStr"/>
+      <c r="D122" s="6" t="inlineStr"/>
       <c r="E122" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3589,31 +3597,23 @@
       </c>
       <c r="F122" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>http://171.244.38.92:7001</t>
+          <t>https://183.81.62.19:443</t>
         </is>
       </c>
       <c r="B123" s="6" t="inlineStr">
         <is>
-          <t>171.244.38.92:7001</t>
-        </is>
-      </c>
-      <c r="C123" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D123" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>183.81.62.19:443</t>
+        </is>
+      </c>
+      <c r="C123" s="6" t="inlineStr"/>
+      <c r="D123" s="6" t="inlineStr"/>
       <c r="E123" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3621,43 +3621,43 @@
       </c>
       <c r="F123" s="6" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
-          <t>http://171.254.93.47:9505</t>
+          <t>https://202.74.59.145</t>
         </is>
       </c>
       <c r="B124" s="6" t="inlineStr">
         <is>
-          <t>171.254.93.47:9505</t>
+          <t>202.74.59.145:443</t>
         </is>
       </c>
       <c r="C124" s="6" t="inlineStr"/>
       <c r="D124" s="6" t="inlineStr"/>
       <c r="E124" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F124" s="6" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>170 Hai Ba Trung, DaKao Ward, District 1, Hochiminh City</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>https://183.81.62.19:443</t>
+          <t>https://203.189.31.24</t>
         </is>
       </c>
       <c r="B125" s="6" t="inlineStr">
         <is>
-          <t>183.81.62.19:443</t>
+          <t>203.189.31.24:443</t>
         </is>
       </c>
       <c r="C125" s="6" t="inlineStr"/>
@@ -3667,21 +3667,17 @@
           <t>Hanoi</t>
         </is>
       </c>
-      <c r="F125" s="6" t="inlineStr">
-        <is>
-          <t>FPT Telecom Company</t>
-        </is>
-      </c>
+      <c r="F125" s="6" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="5" t="inlineStr">
         <is>
-          <t>https://202.74.59.145</t>
+          <t>http://203.205.28.64:8000</t>
         </is>
       </c>
       <c r="B126" s="6" t="inlineStr">
         <is>
-          <t>202.74.59.145:443</t>
+          <t>203.205.28.64:8000</t>
         </is>
       </c>
       <c r="C126" s="6" t="inlineStr"/>
@@ -3693,19 +3689,19 @@
       </c>
       <c r="F126" s="6" t="inlineStr">
         <is>
-          <t>170 Hai Ba Trung, DaKao Ward, District 1, Hochiminh City</t>
+          <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>https://203.189.31.24</t>
+          <t>https://203.205.57.229:443</t>
         </is>
       </c>
       <c r="B127" s="6" t="inlineStr">
         <is>
-          <t>203.189.31.24:443</t>
+          <t>203.205.57.229:443</t>
         </is>
       </c>
       <c r="C127" s="6" t="inlineStr"/>
@@ -3715,45 +3711,65 @@
           <t>Hanoi</t>
         </is>
       </c>
-      <c r="F127" s="6" t="inlineStr"/>
+      <c r="F127" s="6" t="inlineStr">
+        <is>
+          <t>CMC Telecom Infrastructure Company</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
-          <t>http://203.205.28.64:8000</t>
+          <t>http://210.211.98.79:8080</t>
         </is>
       </c>
       <c r="B128" s="6" t="inlineStr">
         <is>
-          <t>203.205.28.64:8000</t>
-        </is>
-      </c>
-      <c r="C128" s="6" t="inlineStr"/>
-      <c r="D128" s="6" t="inlineStr"/>
+          <t>210.211.98.79:8080</t>
+        </is>
+      </c>
+      <c r="C128" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
       <c r="E128" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F128" s="6" t="inlineStr">
         <is>
-          <t>CMC Telecom Infrastructure Company</t>
+          <t>CHT Compamy Ltd</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="5" t="inlineStr">
         <is>
-          <t>https://203.205.57.229:443</t>
+          <t>http://210.211.98.79:8081</t>
         </is>
       </c>
       <c r="B129" s="6" t="inlineStr">
         <is>
-          <t>203.205.57.229:443</t>
-        </is>
-      </c>
-      <c r="C129" s="6" t="inlineStr"/>
-      <c r="D129" s="6" t="inlineStr"/>
+          <t>210.211.98.79:8081</t>
+        </is>
+      </c>
+      <c r="C129" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D129" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
       <c r="E129" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3761,29 +3777,25 @@
       </c>
       <c r="F129" s="6" t="inlineStr">
         <is>
-          <t>CMC Telecom Infrastructure Company</t>
+          <t>CHT Compamy Ltd</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="5" t="inlineStr">
         <is>
-          <t>http://210.211.98.79:8080</t>
+          <t>https://210.211.99.108</t>
         </is>
       </c>
       <c r="B130" s="6" t="inlineStr">
         <is>
-          <t>210.211.98.79:8080</t>
-        </is>
-      </c>
-      <c r="C130" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D130" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
+          <t>210.211.99.108:443</t>
+        </is>
+      </c>
+      <c r="C130" s="6" t="inlineStr"/>
+      <c r="D130" s="6" t="inlineStr">
+        <is>
+          <t>console-403</t>
         </is>
       </c>
       <c r="E130" s="6" t="inlineStr">
@@ -3800,12 +3812,12 @@
     <row r="131">
       <c r="A131" s="5" t="inlineStr">
         <is>
-          <t>http://210.211.98.79:8081</t>
+          <t>http://210.211.99.108:7023</t>
         </is>
       </c>
       <c r="B131" s="6" t="inlineStr">
         <is>
-          <t>210.211.98.79:8081</t>
+          <t>210.211.99.108:7023</t>
         </is>
       </c>
       <c r="C131" s="6" t="inlineStr">
@@ -3813,9 +3825,9 @@
           <t>14.1.1.0.0</t>
         </is>
       </c>
-      <c r="D131" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
+      <c r="D131" s="6" t="inlineStr">
+        <is>
+          <t>console-403;T3-open</t>
         </is>
       </c>
       <c r="E131" s="6" t="inlineStr">
@@ -3832,18 +3844,22 @@
     <row r="132">
       <c r="A132" s="5" t="inlineStr">
         <is>
-          <t>https://210.211.99.108</t>
+          <t>https://210.211.99.108:9023</t>
         </is>
       </c>
       <c r="B132" s="6" t="inlineStr">
         <is>
-          <t>210.211.99.108:443</t>
-        </is>
-      </c>
-      <c r="C132" s="6" t="inlineStr"/>
-      <c r="D132" s="6" t="inlineStr">
-        <is>
-          <t>console-403</t>
+          <t>210.211.99.108:9023</t>
+        </is>
+      </c>
+      <c r="C132" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D132" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
         </is>
       </c>
       <c r="E132" s="6" t="inlineStr">
@@ -3860,12 +3876,12 @@
     <row r="133">
       <c r="A133" s="5" t="inlineStr">
         <is>
-          <t>http://210.211.99.108:7023</t>
+          <t>https://210.211.99.108:9068</t>
         </is>
       </c>
       <c r="B133" s="6" t="inlineStr">
         <is>
-          <t>210.211.99.108:7023</t>
+          <t>210.211.99.108:9068</t>
         </is>
       </c>
       <c r="C133" s="6" t="inlineStr">
@@ -3873,9 +3889,9 @@
           <t>14.1.1.0.0</t>
         </is>
       </c>
-      <c r="D133" s="6" t="inlineStr">
-        <is>
-          <t>console-403;T3-open</t>
+      <c r="D133" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
         </is>
       </c>
       <c r="E133" s="6" t="inlineStr">
@@ -3892,24 +3908,16 @@
     <row r="134">
       <c r="A134" s="5" t="inlineStr">
         <is>
-          <t>https://210.211.99.108:9023</t>
+          <t>https://210.245.45.90</t>
         </is>
       </c>
       <c r="B134" s="6" t="inlineStr">
         <is>
-          <t>210.211.99.108:9023</t>
-        </is>
-      </c>
-      <c r="C134" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D134" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
+          <t>210.245.45.90:443</t>
+        </is>
+      </c>
+      <c r="C134" s="6" t="inlineStr"/>
+      <c r="D134" s="6" t="inlineStr"/>
       <c r="E134" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3917,88 +3925,32 @@
       </c>
       <c r="F134" s="6" t="inlineStr">
         <is>
-          <t>CHT Compamy Ltd</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="5" t="inlineStr">
         <is>
-          <t>https://210.211.99.108:9068</t>
+          <t>https://210.245.119.65</t>
         </is>
       </c>
       <c r="B135" s="6" t="inlineStr">
         <is>
-          <t>210.211.99.108:9068</t>
-        </is>
-      </c>
-      <c r="C135" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D135" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
+          <t>210.245.119.65:443</t>
+        </is>
+      </c>
+      <c r="C135" s="6" t="inlineStr"/>
+      <c r="D135" s="6" t="inlineStr"/>
       <c r="E135" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
         </is>
       </c>
-      <c r="F135" s="6" t="inlineStr">
-        <is>
-          <t>CHT Compamy Ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="5" t="inlineStr">
-        <is>
-          <t>https://210.245.45.90</t>
-        </is>
-      </c>
-      <c r="B136" s="6" t="inlineStr">
-        <is>
-          <t>210.245.45.90:443</t>
-        </is>
-      </c>
-      <c r="C136" s="6" t="inlineStr"/>
-      <c r="D136" s="6" t="inlineStr"/>
-      <c r="E136" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F136" s="6" t="inlineStr">
-        <is>
-          <t>FPT Telecom Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="5" t="inlineStr">
-        <is>
-          <t>https://210.245.119.65</t>
-        </is>
-      </c>
-      <c r="B137" s="6" t="inlineStr">
-        <is>
-          <t>210.245.119.65:443</t>
-        </is>
-      </c>
-      <c r="C137" s="6" t="inlineStr"/>
-      <c r="D137" s="6" t="inlineStr"/>
-      <c r="E137" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F137" s="6" t="inlineStr"/>
+      <c r="F135" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F137"/>
+  <autoFilter ref="A1:F135"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
@@ -4134,8 +4086,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A133" r:id="rId132"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A134" r:id="rId133"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A135" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A136" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A137" r:id="rId136"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
vault backup: 2026-10-09 16:13:06
</commit_message>
<xml_diff>
--- a/WLS-VN-live.xlsx
+++ b/WLS-VN-live.xlsx
@@ -10,7 +10,7 @@
     <sheet name="WLS VN (live)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WLS VN (live)'!$A$1:$F$135</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WLS VN (live)'!$A$1:$F$117</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F135"/>
+  <dimension ref="A1:F117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -636,12 +636,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>http://xbi.xteco.org</t>
+          <t>https://xbi.xteco.org</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>27.71.231.120:80</t>
+          <t>27.71.231.120:443</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
@@ -660,12 +660,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>https://xbi.xteco.org</t>
+          <t>https://rsaweb.mps.gov.vn</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>27.71.231.120:443</t>
+          <t>42.1.75.65:443</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr"/>
@@ -677,19 +677,19 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>CHT Compamy Ltd</t>
+          <t>MOBIFONE Corporation</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>https://rsaweb.mps.gov.vn</t>
+          <t>https://hochieu.xuatnhapcanh.gov.vn</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>42.1.75.65:443</t>
+          <t>42.112.168.100:443</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
@@ -701,19 +701,19 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>MOBIFONE Corporation</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>https://hochieu.xuatnhapcanh.gov.vn</t>
+          <t>https://quanlyluutru.xuatnhapcanh.gov.vn</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>42.112.168.100:443</t>
+          <t>42.112.168.116:443</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr"/>
@@ -732,16 +732,24 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>https://quanlyluutru.xuatnhapcanh.gov.vn</t>
+          <t>https://orabi.kimdental.vn</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>42.112.168.116:443</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr"/>
+          <t>42.115.41.28:443</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>12.2.1.3.0</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -756,24 +764,16 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>https://orabi.kimdental.vn</t>
+          <t>https://dvc.vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>42.115.41.28:443</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>12.2.1.3.0</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
+          <t>45.120.230.40:443</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -781,19 +781,19 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>Creative Communication Vietnam Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>http://dvc.vst.mof.gov.vn</t>
+          <t>https://dvctn.vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.40:80</t>
+          <t>45.120.230.41:443</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
@@ -812,12 +812,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>https://dvc.vst.mof.gov.vn</t>
+          <t>http://vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.40:443</t>
+          <t>45.120.230.45:80</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr"/>
@@ -836,12 +836,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>http://dvctn.vst.mof.gov.vn</t>
+          <t>https://bctcnn.vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.41:80</t>
+          <t>45.120.230.50:443</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
@@ -860,12 +860,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>https://dvctn.vst.mof.gov.vn</t>
+          <t>https://tracuudvc.vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.41:443</t>
+          <t>45.120.230.51:443</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr"/>
@@ -884,12 +884,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>http://vst.mof.gov.vn</t>
+          <t>http://tongcuc.hotrokythuat.asia:8080</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.45:80</t>
+          <t>45.122.253.178:8080</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
@@ -901,43 +901,39 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>http://bctcnn.vst.mof.gov.vn</t>
+          <t>http://dichvucong.danang.vn</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.50:80</t>
+          <t>49.156.52.22:80</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr"/>
       <c r="D18" s="3" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
-        </is>
-      </c>
+          <t>Da Nang</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>https://bctcnn.vst.mof.gov.vn</t>
+          <t>https://pus.customs.gov.vn</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.50:443</t>
+          <t>58.186.80.48:443</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr"/>
@@ -949,19 +945,19 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>http://tracuudvc.vst.mof.gov.vn</t>
+          <t>https://ids.ssc.gov.vn</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.51:80</t>
+          <t>103.3.252.106:443</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr"/>
@@ -973,19 +969,19 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>https://tracuudvc.vst.mof.gov.vn</t>
+          <t>https://congbothongtin.ssc.gov.vn</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.51:443</t>
+          <t>103.3.252.107:443</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr"/>
@@ -997,19 +993,19 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>http://tongcuc.hotrokythuat.asia:8080</t>
+          <t>https://ssc.gov.vn</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>45.122.253.178:8080</t>
+          <t>103.3.252.109:443</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr"/>
@@ -1021,39 +1017,43 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>CMC Telecom Infrastructure Company</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>http://dichvucong.danang.vn</t>
+          <t>https://cims.hnx.vn</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>49.156.52.22:80</t>
+          <t>103.9.212.43:443</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr"/>
       <c r="D23" s="3" t="inlineStr"/>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Da Nang</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr"/>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>HaNoi Stock Exchange</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>http://pus.customs.gov.vn</t>
+          <t>http://hse.vn</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>58.186.80.48:80</t>
+          <t>103.9.212.46:80</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr"/>
@@ -1063,69 +1063,73 @@
           <t>Hanoi</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>FPT Telecom Company</t>
-        </is>
-      </c>
+      <c r="F24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>https://pus.customs.gov.vn</t>
+          <t>https://www.xsmb360.com</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>58.186.80.48:443</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
+          <t>103.82.194.3:443</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Da Nang</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>http://ids.ssc.gov.vn</t>
+          <t>https://idm.homecredit.vn</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>103.3.252.106:80</t>
+          <t>103.111.244.73:443</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr"/>
       <c r="D26" s="3" t="inlineStr"/>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>Home Credit Viet nam Finance Company Limited</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>https://ids.ssc.gov.vn</t>
+          <t>https://www.vinpro.net</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>103.3.252.106:443</t>
+          <t>103.238.209.204:443</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr"/>
@@ -1137,19 +1141,19 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>VINGROUP JOINT STOCK COMPANY</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>http://congbothongtin.ssc.gov.vn</t>
+          <t>https://eoffice.myvnc.com</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>103.3.252.107:80</t>
+          <t>113.160.48.99:443</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr"/>
@@ -1161,215 +1165,259 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>https://congbothongtin.ssc.gov.vn</t>
+          <t>http://apvs1.dlp.com.tw:7001</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>103.3.252.107:443</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
+          <t>113.160.129.228:7001</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Hai Duong</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>https://ssc.gov.vn</t>
+          <t>http://apvs1.dlp.com.tw:9001</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>103.3.252.109:443</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr"/>
-      <c r="D30" s="3" t="inlineStr"/>
+          <t>113.160.129.228:9001</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>T3-open</t>
+        </is>
+      </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Hai Duong</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>http://cims.hnx.vn</t>
+          <t>http://apvs1.dlp.com.tw:9002</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>103.9.212.43:80</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
+          <t>113.160.129.228:9002</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>T3-open</t>
+        </is>
+      </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Hai Duong</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>HaNoi Stock Exchange</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>https://cims.hnx.vn</t>
+          <t>http://www.dtsweb.tech:8081</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>103.9.212.43:443</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr"/>
-      <c r="D32" s="3" t="inlineStr"/>
+          <t>113.161.81.238:8081</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>T3-open</t>
+        </is>
+      </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>HaNoi Stock Exchange</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>http://hse.vn</t>
+          <t>http://www.dtsweb.tech:9001</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>103.9.212.46:80</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr"/>
+          <t>113.161.81.238:9001</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>T3-open</t>
+        </is>
+      </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr"/>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>https://www.xsmb360.com</t>
+          <t>http://www.hddt.agimexpharm.com:8082</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>103.82.194.3:443</t>
+          <t>113.161.212.113:8082</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>T3-open</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Da Nang</t>
+          <t>Long Xuyen</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>http://idm.homecredit.vn</t>
+          <t>http://webdisk.sophattai.com:8080</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>103.111.244.73:80</t>
+          <t>113.185.19.167:8080</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr"/>
       <c r="D35" s="3" t="inlineStr"/>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Home Credit Viet nam Finance Company Limited</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>https://idm.homecredit.vn</t>
+          <t>https://pritos.cloud:3068</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>103.111.244.73:443</t>
+          <t>115.75.20.142:3068</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr"/>
       <c r="D36" s="3" t="inlineStr"/>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Thi Tran Long Dien</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Home Credit Viet nam Finance Company Limited</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>https://www.vinpro.net</t>
+          <t>https://thi.moet.gov.vn</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>103.238.209.204:443</t>
+          <t>115.146.127.162:443</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr"/>
@@ -1379,21 +1427,17 @@
           <t>Hanoi</t>
         </is>
       </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>VINGROUP JOINT STOCK COMPANY</t>
-        </is>
-      </c>
+      <c r="F37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>https://eoffice.myvnc.com</t>
+          <t>http://capcaohcm.toaan.gov.vn</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>113.160.48.99:443</t>
+          <t>123.30.24.180:80</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr"/>
@@ -1412,27 +1456,19 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>http://apvs1.dlp.com.tw:7001</t>
+          <t>https://mla.toaan.gov.vn</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>113.160.129.228:7001</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>123.30.24.180:443</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Hai Duong</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
@@ -1444,27 +1480,19 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>http://apvs1.dlp.com.tw:9001</t>
+          <t>https://cskh.temxacthuc.vn:8081</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>113.160.129.228:9001</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>123.30.208.19:8081</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr"/>
+      <c r="D40" s="3" t="inlineStr"/>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Hai Duong</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -1476,27 +1504,19 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>http://apvs1.dlp.com.tw:9002</t>
+          <t>http://www.topteen.vn</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>113.160.129.228:9002</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>123.30.208.25:80</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr"/>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Hai Duong</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -1508,156 +1528,132 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>http://www.dtsweb.tech:8081</t>
+          <t>http://gmobi.vn</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>113.161.81.238:8081</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>123.31.31.126:80</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr"/>
+      <c r="D42" s="3" t="inlineStr"/>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>http://www.dtsweb.tech:9001</t>
+          <t>http://cskh.temdientu.vn</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>113.161.81.238:9001</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>123.31.41.93:80</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr"/>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>http://www.hddt.agimexpharm.com:8082</t>
+          <t>https://csdlgiaquocgia.mof.gov.vn</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>113.161.212.113:8082</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>182.236.113.46:443</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr"/>
+      <c r="D44" s="3" t="inlineStr"/>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Long Xuyen</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Department of Information Technology and Digital Transformation - Ministry of Finance</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>http://webdisk.sophattai.com:8080</t>
+          <t>https://thongbaotenmien.vn</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>113.185.19.167:8080</t>
+          <t>203.119.73.12:443</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr"/>
       <c r="D45" s="3" t="inlineStr"/>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Vietnam Internet network information center (VNNIC)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>https://pritos.cloud:3068</t>
+          <t>http://qlahs.vksndtc.gov.vn</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>115.75.20.142:3068</t>
+          <t>203.162.255.5:80</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr"/>
       <c r="D46" s="3" t="inlineStr"/>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Thi Tran Long Dien</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>http://thi.moet.gov.vn</t>
+          <t>http://chuyentien.vietinbank.vn</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>115.146.127.162:80</t>
+          <t>203.189.28.86:80</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr"/>
@@ -1667,17 +1663,21 @@
           <t>Hanoi</t>
         </is>
       </c>
-      <c r="F47" s="3" t="inlineStr"/>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>VIETINBANK</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>https://thi.moet.gov.vn</t>
+          <t>https://sso.vietinbank.vn</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>115.146.127.162:443</t>
+          <t>203.189.29.33:443</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr"/>
@@ -1687,45 +1687,57 @@
           <t>Hanoi</t>
         </is>
       </c>
-      <c r="F48" s="3" t="inlineStr"/>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>VIETINBANK-VN</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>http://capcaohcm.toaan.gov.vn</t>
+          <t>https://htttsv.hoasen.edu.vn</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>123.30.24.180:80</t>
+          <t>203.205.57.225:443</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr"/>
       <c r="D49" s="3" t="inlineStr"/>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>https://mla.toaan.gov.vn</t>
+          <t>http://erpbk.hoasen.edu.vn</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>123.30.24.180:443</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr"/>
-      <c r="D50" s="3" t="inlineStr"/>
+          <t>203.205.57.226:80</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>10.3.4.0</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -1733,19 +1745,19 @@
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>https://cskh.temxacthuc.vn:8081</t>
+          <t>http://cms.mebongda.net</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>123.30.208.19:8081</t>
+          <t>210.211.99.108:80</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr"/>
@@ -1757,19 +1769,19 @@
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>CHT Compamy Ltd</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>http://www.topteen.vn</t>
+          <t>http://static.ketquasieutoc.com:8080</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>123.30.208.25:80</t>
+          <t>210.211.99.108:8080</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr"/>
@@ -1781,19 +1793,19 @@
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>CHT Compamy Ltd</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>http://gmobi.vn</t>
+          <t>http://mobilaw.vn</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>123.31.31.126:80</t>
+          <t>210.211.99.130:80</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr"/>
@@ -1803,21 +1815,17 @@
           <t>Hanoi</t>
         </is>
       </c>
-      <c r="F53" s="3" t="inlineStr">
-        <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
-        </is>
-      </c>
+      <c r="F53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>http://cskh.temdientu.vn</t>
+          <t>http://m.xosothongminh.vn</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>123.31.41.93:80</t>
+          <t>210.211.99.133:80</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr"/>
@@ -1827,21 +1835,17 @@
           <t>Hanoi</t>
         </is>
       </c>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
-        </is>
-      </c>
+      <c r="F54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>http://csdlgiaquocgia.mof.gov.vn</t>
+          <t>http://rvt.kenhnhac.vn</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>182.236.113.46:80</t>
+          <t>210.211.99.174:80</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr"/>
@@ -1853,19 +1857,19 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Department of Information Technology and Digital Transformation - Ministry of Finance</t>
+          <t>CHT Compamy Ltd</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>https://csdlgiaquocgia.mof.gov.vn</t>
+          <t>http://dvc-kbnn.fintechviet.vn</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>182.236.113.46:443</t>
+          <t>222.252.98.4:80</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr"/>
@@ -1877,391 +1881,407 @@
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>Department of Information Technology and Digital Transformation - Ministry of Finance</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>http://thongbaotenmien.vn</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>203.119.73.12:80</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr"/>
-      <c r="D57" s="3" t="inlineStr"/>
-      <c r="E57" s="3" t="inlineStr">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>http://14.225.11.33:9001</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>14.225.11.33:9001</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>T3-open</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>http://14.238.41.12:80</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>14.238.41.12:80</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr"/>
+      <c r="D58" s="6" t="inlineStr"/>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>https://14.238.93.114:9184</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>14.238.93.114:9184</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr"/>
+      <c r="D59" s="6" t="inlineStr"/>
+      <c r="E59" s="6" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="F57" s="3" t="inlineStr">
-        <is>
-          <t>Vietnam Internet network information center (VNNIC)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>https://thongbaotenmien.vn</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>203.119.73.12:443</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr"/>
-      <c r="D58" s="3" t="inlineStr"/>
-      <c r="E58" s="3" t="inlineStr">
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>http://14.241.253.96:8081</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>14.241.253.96:8081</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr"/>
+      <c r="D60" s="6" t="inlineStr"/>
+      <c r="E60" s="6" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>Vietnam Internet network information center (VNNIC)</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>http://qlahs.vksndtc.gov.vn</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>203.162.255.5:80</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="inlineStr"/>
-      <c r="D59" s="3" t="inlineStr"/>
-      <c r="E59" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F59" s="3" t="inlineStr">
+      <c r="F60" s="6" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>http://chuyentien.vietinbank.vn</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="inlineStr">
-        <is>
-          <t>203.189.28.86:80</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="inlineStr"/>
-      <c r="D60" s="3" t="inlineStr"/>
-      <c r="E60" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F60" s="3" t="inlineStr">
-        <is>
-          <t>VIETINBANK</t>
-        </is>
-      </c>
-    </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>http://sso.vietinbank.vn</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="inlineStr">
-        <is>
-          <t>203.189.29.33:80</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="inlineStr"/>
-      <c r="D61" s="3" t="inlineStr"/>
-      <c r="E61" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F61" s="3" t="inlineStr">
-        <is>
-          <t>VIETINBANK-VN</t>
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>http://14.241.253.96:8082</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>14.241.253.96:8082</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr"/>
+      <c r="D61" s="6" t="inlineStr"/>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>https://sso.vietinbank.vn</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="inlineStr">
-        <is>
-          <t>203.189.29.33:443</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr"/>
-      <c r="D62" s="3" t="inlineStr"/>
-      <c r="E62" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F62" s="3" t="inlineStr">
-        <is>
-          <t>VIETINBANK-VN</t>
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>https://14.248.84.7:443</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>14.248.84.7:443</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr"/>
+      <c r="D62" s="6" t="inlineStr"/>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>http://htttsv.hoasen.edu.vn</t>
-        </is>
-      </c>
-      <c r="B63" s="3" t="inlineStr">
-        <is>
-          <t>203.205.57.225:80</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="inlineStr"/>
-      <c r="D63" s="3" t="inlineStr"/>
-      <c r="E63" s="3" t="inlineStr">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>http://27.72.123.124:8001</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>27.72.123.124:8001</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr"/>
+      <c r="D63" s="6" t="inlineStr"/>
+      <c r="E63" s="6" t="inlineStr">
+        <is>
+          <t>Sa Pa</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>Viettel Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>http://27.72.123.124:8003</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>27.72.123.124:8003</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr"/>
+      <c r="D64" s="6" t="inlineStr"/>
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t>Ha Long</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>Viettel Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>https://42.115.41.27:443</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>42.115.41.27:443</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr"/>
+      <c r="D65" s="6" t="inlineStr"/>
+      <c r="E65" s="6" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="F63" s="3" t="inlineStr">
-        <is>
-          <t>CMC Telecom Infrastructure Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>https://htttsv.hoasen.edu.vn</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>203.205.57.225:443</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr"/>
-      <c r="D64" s="3" t="inlineStr"/>
-      <c r="E64" s="3" t="inlineStr">
+      <c r="F65" s="6" t="inlineStr">
+        <is>
+          <t>FPT Telecom Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>http://42.118.60.193:7001</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>42.118.60.193:7001</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>FPT Telecom Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>https://45.120.230.45</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>45.120.230.45:443</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr"/>
+      <c r="D67" s="6" t="inlineStr"/>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>Creative Communication Vietnam Joint Stock Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>http://49.213.88.170:7001</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>49.213.88.170:7001</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="F64" s="3" t="inlineStr">
-        <is>
-          <t>CMC Telecom Infrastructure Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>http://erpbk.hoasen.edu.vn</t>
-        </is>
-      </c>
-      <c r="B65" s="3" t="inlineStr">
-        <is>
-          <t>203.205.57.226:80</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="inlineStr">
-        <is>
-          <t>10.3.4.0</t>
-        </is>
-      </c>
-      <c r="D65" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
-      <c r="E65" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F65" s="3" t="inlineStr">
-        <is>
-          <t>CMC Telecom Infrastructure Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>http://cms.mebongda.net</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>210.211.99.108:80</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="inlineStr"/>
-      <c r="D66" s="3" t="inlineStr"/>
-      <c r="E66" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F66" s="3" t="inlineStr">
-        <is>
-          <t>CHT Compamy Ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>http://static.ketquasieutoc.com:8080</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>210.211.99.108:8080</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="inlineStr"/>
-      <c r="D67" s="3" t="inlineStr"/>
-      <c r="E67" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="inlineStr">
-        <is>
-          <t>CHT Compamy Ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>http://mobilaw.vn</t>
-        </is>
-      </c>
-      <c r="B68" s="3" t="inlineStr">
-        <is>
-          <t>210.211.99.130:80</t>
-        </is>
-      </c>
-      <c r="C68" s="3" t="inlineStr"/>
-      <c r="D68" s="3" t="inlineStr"/>
-      <c r="E68" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F68" s="3" t="inlineStr"/>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>VNG Corporation</t>
+        </is>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>http://m.xosothongminh.vn</t>
-        </is>
-      </c>
-      <c r="B69" s="3" t="inlineStr">
-        <is>
-          <t>210.211.99.133:80</t>
-        </is>
-      </c>
-      <c r="C69" s="3" t="inlineStr"/>
-      <c r="D69" s="3" t="inlineStr"/>
-      <c r="E69" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F69" s="3" t="inlineStr"/>
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>https://103.3.252.106:7002</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>103.3.252.106:7002</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr"/>
+      <c r="D69" s="6" t="inlineStr"/>
+      <c r="E69" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>http://rvt.kenhnhac.vn</t>
-        </is>
-      </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>210.211.99.174:80</t>
-        </is>
-      </c>
-      <c r="C70" s="3" t="inlineStr"/>
-      <c r="D70" s="3" t="inlineStr"/>
-      <c r="E70" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F70" s="3" t="inlineStr">
-        <is>
-          <t>CHT Compamy Ltd</t>
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>https://103.3.252.107:7002</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>103.3.252.107:7002</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr"/>
+      <c r="D70" s="6" t="inlineStr"/>
+      <c r="E70" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>http://dvc-kbnn.fintechviet.vn</t>
-        </is>
-      </c>
-      <c r="B71" s="3" t="inlineStr">
-        <is>
-          <t>222.252.98.4:80</t>
-        </is>
-      </c>
-      <c r="C71" s="3" t="inlineStr"/>
-      <c r="D71" s="3" t="inlineStr"/>
-      <c r="E71" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F71" s="3" t="inlineStr">
-        <is>
-          <t>VNPT Corp</t>
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>http://103.3.252.109:80</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>103.3.252.109:80</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr"/>
+      <c r="D71" s="6" t="inlineStr"/>
+      <c r="E71" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>http://14.225.11.33:9001</t>
+          <t>http://103.3.252.133</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>14.225.11.33:9001</t>
-        </is>
-      </c>
-      <c r="C72" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D72" s="6" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>103.3.252.133:80</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr"/>
+      <c r="D72" s="6" t="inlineStr"/>
       <c r="E72" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -2269,19 +2289,19 @@
       </c>
       <c r="F72" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>http://14.238.41.12:80</t>
+          <t>http://103.9.213.43</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>14.238.41.12:80</t>
+          <t>103.9.213.43:80</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr"/>
@@ -2293,74 +2313,94 @@
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>HaNoi Stock Exchange</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>https://14.238.93.114:9184</t>
+          <t>https://103.82.192.168</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>14.238.93.114:9184</t>
-        </is>
-      </c>
-      <c r="C74" s="6" t="inlineStr"/>
-      <c r="D74" s="6" t="inlineStr"/>
+          <t>103.82.192.168:443</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Da Nang</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>CLOUDFLY CORPORATION</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>http://14.241.253.96:8081</t>
+          <t>http://103.82.194.3</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>14.241.253.96:8081</t>
-        </is>
-      </c>
-      <c r="C75" s="6" t="inlineStr"/>
-      <c r="D75" s="6" t="inlineStr"/>
+          <t>103.82.194.3:80</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Da Nang</t>
         </is>
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>http://14.241.253.96:8082</t>
+          <t>https://103.120.242.145:8081</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>14.241.253.96:8082</t>
+          <t>103.120.242.145:8081</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr"/>
-      <c r="D76" s="6" t="inlineStr"/>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>console-403</t>
+        </is>
+      </c>
       <c r="E76" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F76" s="6" t="inlineStr">
@@ -2372,84 +2412,80 @@
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>https://14.248.84.7:443</t>
+          <t>http://103.146.20.88:443</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>14.248.84.7:443</t>
+          <t>103.146.20.88:443</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr"/>
       <c r="D77" s="6" t="inlineStr"/>
-      <c r="E77" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="E77" s="6" t="inlineStr"/>
       <c r="F77" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>International Distribution Corporation</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>http://27.72.123.124:8001</t>
+          <t>https://103.150.240.14:443</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>27.72.123.124:8001</t>
+          <t>103.150.240.14:443</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr"/>
       <c r="D78" s="6" t="inlineStr"/>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>Sa Pa</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F78" s="6" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>INTELLIGENCE INFORMATION SYSTEM CO, LTD</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>http://27.72.123.124:8003</t>
+          <t>https://103.238.209.174</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>27.72.123.124:8003</t>
+          <t>103.238.209.174:443</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr"/>
       <c r="D79" s="6" t="inlineStr"/>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>Ha Long</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F79" s="6" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>VINGROUP JOINT STOCK COMPANY</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>https://42.115.41.27:443</t>
+          <t>https://112.109.89.131</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>42.115.41.27:443</t>
+          <t>112.109.89.131:443</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr"/>
@@ -2461,31 +2497,23 @@
       </c>
       <c r="F80" s="6" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>Minh Tu Telecom Limited Company</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>http://42.118.60.193:7001</t>
+          <t>http://113.160.181.154:8001</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>42.118.60.193:7001</t>
-        </is>
-      </c>
-      <c r="C81" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D81" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>113.160.181.154:8001</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr"/>
+      <c r="D81" s="6" t="inlineStr"/>
       <c r="E81" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -2493,53 +2521,61 @@
       </c>
       <c r="F81" s="6" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>https://45.120.230.45</t>
+          <t>http://113.160.201.159:7001</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>45.120.230.45:443</t>
-        </is>
-      </c>
-      <c r="C82" s="6" t="inlineStr"/>
-      <c r="D82" s="6" t="inlineStr"/>
+          <t>113.160.201.159:7001</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
       <c r="E82" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Thai Binh</t>
         </is>
       </c>
       <c r="F82" s="6" t="inlineStr">
         <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>http://49.213.88.170:7001</t>
+          <t>http://113.161.43.248:9001</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>49.213.88.170:7001</t>
+          <t>113.161.43.248:9001</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D83" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
+          <t>14.1.2.0.0</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>T3-open</t>
         </is>
       </c>
       <c r="E83" s="6" t="inlineStr">
@@ -2549,43 +2585,51 @@
       </c>
       <c r="F83" s="6" t="inlineStr">
         <is>
-          <t>VNG Corporation</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>https://103.3.252.106:7002</t>
+          <t>http://113.163.187.3:27001</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>103.3.252.106:7002</t>
-        </is>
-      </c>
-      <c r="C84" s="6" t="inlineStr"/>
-      <c r="D84" s="6" t="inlineStr"/>
+          <t>113.163.187.3:27001</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
       <c r="E84" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Phan Rang-Thap Cham</t>
         </is>
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>https://103.3.252.107:7002</t>
+          <t>http://113.185.0.60:8080</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>103.3.252.107:7002</t>
+          <t>113.185.0.60:8080</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr"/>
@@ -2597,23 +2641,31 @@
       </c>
       <c r="F85" s="6" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>http://103.3.252.109:80</t>
+          <t>http://117.4.32.40:1111</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>103.3.252.109:80</t>
-        </is>
-      </c>
-      <c r="C86" s="6" t="inlineStr"/>
-      <c r="D86" s="6" t="inlineStr"/>
+          <t>117.4.32.40:1111</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
       <c r="E86" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -2621,23 +2673,31 @@
       </c>
       <c r="F86" s="6" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>http://103.3.252.133</t>
+          <t>http://117.4.241.247:1112</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>103.3.252.133:80</t>
-        </is>
-      </c>
-      <c r="C87" s="6" t="inlineStr"/>
-      <c r="D87" s="6" t="inlineStr"/>
+          <t>117.4.241.247:1112</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
       <c r="E87" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -2645,145 +2705,133 @@
       </c>
       <c r="F87" s="6" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>http://103.9.213.43</t>
+          <t>https://118.69.32.193:3068</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>103.9.213.43:80</t>
+          <t>118.69.32.193:3068</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr"/>
       <c r="D88" s="6" t="inlineStr"/>
       <c r="E88" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Thu Dau Mot</t>
         </is>
       </c>
       <c r="F88" s="6" t="inlineStr">
         <is>
-          <t>HaNoi Stock Exchange</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>http://103.82.192.168</t>
+          <t>http://118.69.182.224:9079</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>103.82.192.168:80</t>
+          <t>118.69.182.224:9079</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D89" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D89" s="6" t="inlineStr">
+        <is>
+          <t>T3-open</t>
         </is>
       </c>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t>Da Nang</t>
+          <t>Bien Hoa</t>
         </is>
       </c>
       <c r="F89" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>https://103.82.192.168</t>
+          <t>http://123.30.208.19:80</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>103.82.192.168:443</t>
-        </is>
-      </c>
-      <c r="C90" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D90" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
+          <t>123.30.208.19:80</t>
+        </is>
+      </c>
+      <c r="C90" s="6" t="inlineStr"/>
+      <c r="D90" s="6" t="inlineStr"/>
       <c r="E90" s="6" t="inlineStr">
         <is>
-          <t>Da Nang</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F90" s="6" t="inlineStr">
         <is>
-          <t>CLOUDFLY CORPORATION</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>http://103.82.194.3</t>
+          <t>https://123.30.208.19:443</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>103.82.194.3:80</t>
-        </is>
-      </c>
-      <c r="C91" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D91" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
+          <t>123.30.208.19:443</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="inlineStr"/>
+      <c r="D91" s="6" t="inlineStr"/>
       <c r="E91" s="6" t="inlineStr">
         <is>
-          <t>Da Nang</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F91" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>https://103.120.242.145:8081</t>
+          <t>http://123.31.31.119:49163</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>103.120.242.145:8081</t>
-        </is>
-      </c>
-      <c r="C92" s="6" t="inlineStr"/>
-      <c r="D92" s="6" t="inlineStr">
-        <is>
-          <t>console-403</t>
+          <t>123.31.31.119:49163</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
         </is>
       </c>
       <c r="E92" s="6" t="inlineStr">
@@ -2793,67 +2841,87 @@
       </c>
       <c r="F92" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>http://103.146.20.88:443</t>
+          <t>http://123.31.31.125:49163</t>
         </is>
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>103.146.20.88:443</t>
-        </is>
-      </c>
-      <c r="C93" s="6" t="inlineStr"/>
-      <c r="D93" s="6" t="inlineStr"/>
-      <c r="E93" s="6" t="inlineStr"/>
+          <t>123.31.31.125:49163</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
+      <c r="E93" s="6" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
       <c r="F93" s="6" t="inlineStr">
         <is>
-          <t>International Distribution Corporation</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>https://103.150.240.14:443</t>
+          <t>https://123.31.36.60</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>103.150.240.14:443</t>
+          <t>123.31.36.60:443</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr"/>
       <c r="D94" s="6" t="inlineStr"/>
       <c r="E94" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F94" s="6" t="inlineStr">
         <is>
-          <t>INTELLIGENCE INFORMATION SYSTEM CO, LTD</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>http://103.238.209.174</t>
+          <t>http://123.31.36.63:8002</t>
         </is>
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>103.238.209.174:80</t>
-        </is>
-      </c>
-      <c r="C95" s="6" t="inlineStr"/>
-      <c r="D95" s="6" t="inlineStr"/>
+          <t>123.31.36.63:8002</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -2861,67 +2929,67 @@
       </c>
       <c r="F95" s="6" t="inlineStr">
         <is>
-          <t>VINGROUP JOINT STOCK COMPANY</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>https://103.238.209.174</t>
+          <t>https://124.158.11.115:8443</t>
         </is>
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>103.238.209.174:443</t>
+          <t>124.158.11.115:8443</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr"/>
       <c r="D96" s="6" t="inlineStr"/>
       <c r="E96" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F96" s="6" t="inlineStr">
         <is>
-          <t>VINGROUP JOINT STOCK COMPANY</t>
+          <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>https://112.109.89.131</t>
+          <t>https://144.48.24.66:5620</t>
         </is>
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>112.109.89.131:443</t>
+          <t>144.48.24.66:5620</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr"/>
       <c r="D97" s="6" t="inlineStr"/>
       <c r="E97" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F97" s="6" t="inlineStr">
         <is>
-          <t>Minh Tu Telecom Limited Company</t>
+          <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>http://113.160.181.154:8001</t>
+          <t>https://144.48.24.66:5650</t>
         </is>
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>113.160.181.154:8001</t>
+          <t>144.48.24.66:5650</t>
         </is>
       </c>
       <c r="C98" s="6" t="inlineStr"/>
@@ -2933,119 +3001,103 @@
       </c>
       <c r="F98" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>http://113.160.201.159:7001</t>
+          <t>https://144.48.24.66:5680</t>
         </is>
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>113.160.201.159:7001</t>
-        </is>
-      </c>
-      <c r="C99" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D99" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>144.48.24.66:5680</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="inlineStr"/>
+      <c r="D99" s="6" t="inlineStr"/>
       <c r="E99" s="6" t="inlineStr">
         <is>
-          <t>Thai Binh</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F99" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>http://113.161.43.248:9001</t>
+          <t>https://144.48.24.69:5620</t>
         </is>
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
-          <t>113.161.43.248:9001</t>
-        </is>
-      </c>
-      <c r="C100" s="6" t="inlineStr">
-        <is>
-          <t>14.1.2.0.0</t>
-        </is>
-      </c>
-      <c r="D100" s="6" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>144.48.24.69:5620</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="inlineStr"/>
+      <c r="D100" s="6" t="inlineStr"/>
       <c r="E100" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F100" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>http://113.163.187.3:27001</t>
+          <t>https://144.48.24.69:5650</t>
         </is>
       </c>
       <c r="B101" s="6" t="inlineStr">
         <is>
-          <t>113.163.187.3:27001</t>
-        </is>
-      </c>
-      <c r="C101" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D101" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>144.48.24.69:5650</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="inlineStr"/>
+      <c r="D101" s="6" t="inlineStr"/>
       <c r="E101" s="6" t="inlineStr">
         <is>
-          <t>Phan Rang-Thap Cham</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F101" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>http://113.185.0.60:8080</t>
+          <t>http://160.191.101.129:9001</t>
         </is>
       </c>
       <c r="B102" s="6" t="inlineStr">
         <is>
-          <t>113.185.0.60:8080</t>
-        </is>
-      </c>
-      <c r="C102" s="6" t="inlineStr"/>
-      <c r="D102" s="6" t="inlineStr"/>
+          <t>160.191.101.129:9001</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>14.1.2.0.0</t>
+        </is>
+      </c>
+      <c r="D102" s="6" t="inlineStr">
+        <is>
+          <t>T3-open</t>
+        </is>
+      </c>
       <c r="E102" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3053,19 +3105,19 @@
       </c>
       <c r="F102" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>http://117.4.32.40:1111</t>
+          <t>http://171.244.38.92:7001</t>
         </is>
       </c>
       <c r="B103" s="6" t="inlineStr">
         <is>
-          <t>117.4.32.40:1111</t>
+          <t>171.244.38.92:7001</t>
         </is>
       </c>
       <c r="C103" s="6" t="inlineStr">
@@ -3092,24 +3144,16 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>http://117.4.241.247:1112</t>
+          <t>http://171.254.93.47:9505</t>
         </is>
       </c>
       <c r="B104" s="6" t="inlineStr">
         <is>
-          <t>117.4.241.247:1112</t>
-        </is>
-      </c>
-      <c r="C104" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D104" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>171.254.93.47:9505</t>
+        </is>
+      </c>
+      <c r="C104" s="6" t="inlineStr"/>
+      <c r="D104" s="6" t="inlineStr"/>
       <c r="E104" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3124,19 +3168,19 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>https://118.69.32.193:3068</t>
+          <t>https://183.81.62.19:443</t>
         </is>
       </c>
       <c r="B105" s="6" t="inlineStr">
         <is>
-          <t>118.69.32.193:3068</t>
+          <t>183.81.62.19:443</t>
         </is>
       </c>
       <c r="C105" s="6" t="inlineStr"/>
       <c r="D105" s="6" t="inlineStr"/>
       <c r="E105" s="6" t="inlineStr">
         <is>
-          <t>Thu Dau Mot</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F105" s="6" t="inlineStr">
@@ -3148,44 +3192,36 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>http://118.69.182.224:9079</t>
+          <t>https://202.74.59.145</t>
         </is>
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>118.69.182.224:9079</t>
-        </is>
-      </c>
-      <c r="C106" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D106" s="6" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
+          <t>202.74.59.145:443</t>
+        </is>
+      </c>
+      <c r="C106" s="6" t="inlineStr"/>
+      <c r="D106" s="6" t="inlineStr"/>
       <c r="E106" s="6" t="inlineStr">
         <is>
-          <t>Bien Hoa</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F106" s="6" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>170 Hai Ba Trung, DaKao Ward, District 1, Hochiminh City</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>http://123.30.208.19:80</t>
+          <t>https://203.189.31.24</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>123.30.208.19:80</t>
+          <t>203.189.31.24:443</t>
         </is>
       </c>
       <c r="C107" s="6" t="inlineStr"/>
@@ -3195,57 +3231,45 @@
           <t>Hanoi</t>
         </is>
       </c>
-      <c r="F107" s="6" t="inlineStr">
-        <is>
-          <t>VNPT Corp</t>
-        </is>
-      </c>
+      <c r="F107" s="6" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>https://123.30.208.19:443</t>
+          <t>http://203.205.28.64:8000</t>
         </is>
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>123.30.208.19:443</t>
+          <t>203.205.28.64:8000</t>
         </is>
       </c>
       <c r="C108" s="6" t="inlineStr"/>
       <c r="D108" s="6" t="inlineStr"/>
       <c r="E108" s="6" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="F108" s="6" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>http://123.31.31.119:49163</t>
+          <t>https://203.205.57.229:443</t>
         </is>
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>123.31.31.119:49163</t>
-        </is>
-      </c>
-      <c r="C109" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D109" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
+          <t>203.205.57.229:443</t>
+        </is>
+      </c>
+      <c r="C109" s="6" t="inlineStr"/>
+      <c r="D109" s="6" t="inlineStr"/>
       <c r="E109" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3253,19 +3277,19 @@
       </c>
       <c r="F109" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>CMC Telecom Infrastructure Company</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>http://123.31.31.125:49163</t>
+          <t>http://210.211.98.79:8080</t>
         </is>
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>123.31.31.125:49163</t>
+          <t>210.211.98.79:8080</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
@@ -3275,7 +3299,7 @@
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>console-open;T3-open</t>
+          <t>console-open</t>
         </is>
       </c>
       <c r="E110" s="6" t="inlineStr">
@@ -3285,23 +3309,31 @@
       </c>
       <c r="F110" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>CHT Compamy Ltd</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>http://123.31.36.60</t>
+          <t>http://210.211.98.79:8081</t>
         </is>
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>123.31.36.60:80</t>
-        </is>
-      </c>
-      <c r="C111" s="6" t="inlineStr"/>
-      <c r="D111" s="6" t="inlineStr"/>
+          <t>210.211.98.79:8081</t>
+        </is>
+      </c>
+      <c r="C111" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>console-open;T3-open</t>
+        </is>
+      </c>
       <c r="E111" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3309,23 +3341,27 @@
       </c>
       <c r="F111" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>CHT Compamy Ltd</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
         <is>
-          <t>https://123.31.36.60</t>
+          <t>https://210.211.99.108</t>
         </is>
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>123.31.36.60:443</t>
+          <t>210.211.99.108:443</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr"/>
-      <c r="D112" s="6" t="inlineStr"/>
+      <c r="D112" s="6" t="inlineStr">
+        <is>
+          <t>console-403</t>
+        </is>
+      </c>
       <c r="E112" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3333,19 +3369,19 @@
       </c>
       <c r="F112" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>CHT Compamy Ltd</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>http://123.31.36.63:8002</t>
+          <t>http://210.211.99.108:7023</t>
         </is>
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>123.31.36.63:8002</t>
+          <t>210.211.99.108:7023</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
@@ -3353,9 +3389,9 @@
           <t>14.1.1.0.0</t>
         </is>
       </c>
-      <c r="D113" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
+      <c r="D113" s="6" t="inlineStr">
+        <is>
+          <t>console-403;T3-open</t>
         </is>
       </c>
       <c r="E113" s="6" t="inlineStr">
@@ -3365,47 +3401,63 @@
       </c>
       <c r="F113" s="6" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>CHT Compamy Ltd</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="5" t="inlineStr">
         <is>
-          <t>https://124.158.11.115:8443</t>
+          <t>https://210.211.99.108:9023</t>
         </is>
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>124.158.11.115:8443</t>
-        </is>
-      </c>
-      <c r="C114" s="6" t="inlineStr"/>
-      <c r="D114" s="6" t="inlineStr"/>
+          <t>210.211.99.108:9023</t>
+        </is>
+      </c>
+      <c r="C114" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
       <c r="E114" s="6" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="F114" s="6" t="inlineStr">
         <is>
-          <t>CMC Telecom Infrastructure Company</t>
+          <t>CHT Compamy Ltd</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>https://144.48.24.66:5620</t>
+          <t>https://210.211.99.108:9068</t>
         </is>
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>144.48.24.66:5620</t>
-        </is>
-      </c>
-      <c r="C115" s="6" t="inlineStr"/>
-      <c r="D115" s="6" t="inlineStr"/>
+          <t>210.211.99.108:9068</t>
+        </is>
+      </c>
+      <c r="C115" s="6" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>console-open</t>
+        </is>
+      </c>
       <c r="E115" s="6" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -3413,19 +3465,19 @@
       </c>
       <c r="F115" s="6" t="inlineStr">
         <is>
-          <t>CMC Telecom Infrastructure Company</t>
+          <t>CHT Compamy Ltd</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>https://144.48.24.66:5650</t>
+          <t>https://210.245.45.90</t>
         </is>
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
-          <t>144.48.24.66:5650</t>
+          <t>210.245.45.90:443</t>
         </is>
       </c>
       <c r="C116" s="6" t="inlineStr"/>
@@ -3437,19 +3489,19 @@
       </c>
       <c r="F116" s="6" t="inlineStr">
         <is>
-          <t>CMC Telecom Infrastructure Company</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>https://144.48.24.66:5680</t>
+          <t>https://210.245.119.65</t>
         </is>
       </c>
       <c r="B117" s="6" t="inlineStr">
         <is>
-          <t>144.48.24.66:5680</t>
+          <t>210.245.119.65:443</t>
         </is>
       </c>
       <c r="C117" s="6" t="inlineStr"/>
@@ -3459,498 +3511,10 @@
           <t>Hanoi</t>
         </is>
       </c>
-      <c r="F117" s="6" t="inlineStr">
-        <is>
-          <t>CMC Telecom Infrastructure Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="5" t="inlineStr">
-        <is>
-          <t>https://144.48.24.69:5620</t>
-        </is>
-      </c>
-      <c r="B118" s="6" t="inlineStr">
-        <is>
-          <t>144.48.24.69:5620</t>
-        </is>
-      </c>
-      <c r="C118" s="6" t="inlineStr"/>
-      <c r="D118" s="6" t="inlineStr"/>
-      <c r="E118" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F118" s="6" t="inlineStr">
-        <is>
-          <t>CMC Telecom Infrastructure Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="5" t="inlineStr">
-        <is>
-          <t>https://144.48.24.69:5650</t>
-        </is>
-      </c>
-      <c r="B119" s="6" t="inlineStr">
-        <is>
-          <t>144.48.24.69:5650</t>
-        </is>
-      </c>
-      <c r="C119" s="6" t="inlineStr"/>
-      <c r="D119" s="6" t="inlineStr"/>
-      <c r="E119" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F119" s="6" t="inlineStr">
-        <is>
-          <t>CMC Telecom Infrastructure Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="5" t="inlineStr">
-        <is>
-          <t>http://160.191.101.129:9001</t>
-        </is>
-      </c>
-      <c r="B120" s="6" t="inlineStr">
-        <is>
-          <t>160.191.101.129:9001</t>
-        </is>
-      </c>
-      <c r="C120" s="6" t="inlineStr">
-        <is>
-          <t>14.1.2.0.0</t>
-        </is>
-      </c>
-      <c r="D120" s="6" t="inlineStr">
-        <is>
-          <t>T3-open</t>
-        </is>
-      </c>
-      <c r="E120" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F120" s="6" t="inlineStr">
-        <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="5" t="inlineStr">
-        <is>
-          <t>http://171.244.38.92:7001</t>
-        </is>
-      </c>
-      <c r="B121" s="6" t="inlineStr">
-        <is>
-          <t>171.244.38.92:7001</t>
-        </is>
-      </c>
-      <c r="C121" s="6" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D121" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
-      <c r="E121" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F121" s="6" t="inlineStr">
-        <is>
-          <t>Viettel Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="5" t="inlineStr">
-        <is>
-          <t>http://171.254.93.47:9505</t>
-        </is>
-      </c>
-      <c r="B122" s="6" t="inlineStr">
-        <is>
-          <t>171.254.93.47:9505</t>
-        </is>
-      </c>
-      <c r="C122" s="6" t="inlineStr"/>
-      <c r="D122" s="6" t="inlineStr"/>
-      <c r="E122" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F122" s="6" t="inlineStr">
-        <is>
-          <t>Viettel Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="5" t="inlineStr">
-        <is>
-          <t>https://183.81.62.19:443</t>
-        </is>
-      </c>
-      <c r="B123" s="6" t="inlineStr">
-        <is>
-          <t>183.81.62.19:443</t>
-        </is>
-      </c>
-      <c r="C123" s="6" t="inlineStr"/>
-      <c r="D123" s="6" t="inlineStr"/>
-      <c r="E123" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F123" s="6" t="inlineStr">
-        <is>
-          <t>FPT Telecom Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="5" t="inlineStr">
-        <is>
-          <t>https://202.74.59.145</t>
-        </is>
-      </c>
-      <c r="B124" s="6" t="inlineStr">
-        <is>
-          <t>202.74.59.145:443</t>
-        </is>
-      </c>
-      <c r="C124" s="6" t="inlineStr"/>
-      <c r="D124" s="6" t="inlineStr"/>
-      <c r="E124" s="6" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
-      <c r="F124" s="6" t="inlineStr">
-        <is>
-          <t>170 Hai Ba Trung, DaKao Ward, District 1, Hochiminh City</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="5" t="inlineStr">
-        <is>
-          <t>https://203.189.31.24</t>
-        </is>
-      </c>
-      <c r="B125" s="6" t="inlineStr">
-        <is>
-          <t>203.189.31.24:443</t>
-        </is>
-      </c>
-      <c r="C125" s="6" t="inlineStr"/>
-      <c r="D125" s="6" t="inlineStr"/>
-      <c r="E125" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F125" s="6" t="inlineStr"/>
-    </row>
-    <row r="126">
-      <c r="A126" s="5" t="inlineStr">
-        <is>
-          <t>http://203.205.28.64:8000</t>
-        </is>
-      </c>
-      <c r="B126" s="6" t="inlineStr">
-        <is>
-          <t>203.205.28.64:8000</t>
-        </is>
-      </c>
-      <c r="C126" s="6" t="inlineStr"/>
-      <c r="D126" s="6" t="inlineStr"/>
-      <c r="E126" s="6" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
-      <c r="F126" s="6" t="inlineStr">
-        <is>
-          <t>CMC Telecom Infrastructure Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="5" t="inlineStr">
-        <is>
-          <t>https://203.205.57.229:443</t>
-        </is>
-      </c>
-      <c r="B127" s="6" t="inlineStr">
-        <is>
-          <t>203.205.57.229:443</t>
-        </is>
-      </c>
-      <c r="C127" s="6" t="inlineStr"/>
-      <c r="D127" s="6" t="inlineStr"/>
-      <c r="E127" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F127" s="6" t="inlineStr">
-        <is>
-          <t>CMC Telecom Infrastructure Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="5" t="inlineStr">
-        <is>
-          <t>http://210.211.98.79:8080</t>
-        </is>
-      </c>
-      <c r="B128" s="6" t="inlineStr">
-        <is>
-          <t>210.211.98.79:8080</t>
-        </is>
-      </c>
-      <c r="C128" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D128" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
-      <c r="E128" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F128" s="6" t="inlineStr">
-        <is>
-          <t>CHT Compamy Ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="5" t="inlineStr">
-        <is>
-          <t>http://210.211.98.79:8081</t>
-        </is>
-      </c>
-      <c r="B129" s="6" t="inlineStr">
-        <is>
-          <t>210.211.98.79:8081</t>
-        </is>
-      </c>
-      <c r="C129" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D129" s="4" t="inlineStr">
-        <is>
-          <t>console-open;T3-open</t>
-        </is>
-      </c>
-      <c r="E129" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F129" s="6" t="inlineStr">
-        <is>
-          <t>CHT Compamy Ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="5" t="inlineStr">
-        <is>
-          <t>https://210.211.99.108</t>
-        </is>
-      </c>
-      <c r="B130" s="6" t="inlineStr">
-        <is>
-          <t>210.211.99.108:443</t>
-        </is>
-      </c>
-      <c r="C130" s="6" t="inlineStr"/>
-      <c r="D130" s="6" t="inlineStr">
-        <is>
-          <t>console-403</t>
-        </is>
-      </c>
-      <c r="E130" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F130" s="6" t="inlineStr">
-        <is>
-          <t>CHT Compamy Ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="5" t="inlineStr">
-        <is>
-          <t>http://210.211.99.108:7023</t>
-        </is>
-      </c>
-      <c r="B131" s="6" t="inlineStr">
-        <is>
-          <t>210.211.99.108:7023</t>
-        </is>
-      </c>
-      <c r="C131" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D131" s="6" t="inlineStr">
-        <is>
-          <t>console-403;T3-open</t>
-        </is>
-      </c>
-      <c r="E131" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F131" s="6" t="inlineStr">
-        <is>
-          <t>CHT Compamy Ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="5" t="inlineStr">
-        <is>
-          <t>https://210.211.99.108:9023</t>
-        </is>
-      </c>
-      <c r="B132" s="6" t="inlineStr">
-        <is>
-          <t>210.211.99.108:9023</t>
-        </is>
-      </c>
-      <c r="C132" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D132" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
-      <c r="E132" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F132" s="6" t="inlineStr">
-        <is>
-          <t>CHT Compamy Ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="5" t="inlineStr">
-        <is>
-          <t>https://210.211.99.108:9068</t>
-        </is>
-      </c>
-      <c r="B133" s="6" t="inlineStr">
-        <is>
-          <t>210.211.99.108:9068</t>
-        </is>
-      </c>
-      <c r="C133" s="6" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D133" s="4" t="inlineStr">
-        <is>
-          <t>console-open</t>
-        </is>
-      </c>
-      <c r="E133" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F133" s="6" t="inlineStr">
-        <is>
-          <t>CHT Compamy Ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="5" t="inlineStr">
-        <is>
-          <t>https://210.245.45.90</t>
-        </is>
-      </c>
-      <c r="B134" s="6" t="inlineStr">
-        <is>
-          <t>210.245.45.90:443</t>
-        </is>
-      </c>
-      <c r="C134" s="6" t="inlineStr"/>
-      <c r="D134" s="6" t="inlineStr"/>
-      <c r="E134" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F134" s="6" t="inlineStr">
-        <is>
-          <t>FPT Telecom Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="5" t="inlineStr">
-        <is>
-          <t>https://210.245.119.65</t>
-        </is>
-      </c>
-      <c r="B135" s="6" t="inlineStr">
-        <is>
-          <t>210.245.119.65:443</t>
-        </is>
-      </c>
-      <c r="C135" s="6" t="inlineStr"/>
-      <c r="D135" s="6" t="inlineStr"/>
-      <c r="E135" s="6" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="F135" s="6" t="inlineStr"/>
+      <c r="F117" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F135"/>
+  <autoFilter ref="A1:F117"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
@@ -4068,24 +3632,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A115" r:id="rId114"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A116" r:id="rId115"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A117" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A118" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A119" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A120" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A121" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A122" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A123" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A124" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A125" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A126" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A127" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A128" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A129" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A130" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A131" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A132" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A133" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A134" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A135" r:id="rId134"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>